<commit_message>
excel fixes after error checking script
</commit_message>
<xml_diff>
--- a/Excel/4_7_ManureManagement_OtherLivestock_WIP_v01.xlsx
+++ b/Excel/4_7_ManureManagement_OtherLivestock_WIP_v01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7D09803-948D-4888-B134-CC271036A0AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21E7F8F4-33AE-4C1B-AC3E-FA16368EE32F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="36255" windowHeight="19140" firstSheet="8" activeTab="11" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="390" yWindow="390" windowWidth="36255" windowHeight="19140" firstSheet="8" activeTab="8" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="71" r:id="rId1"/>
@@ -29292,7 +29292,7 @@
         <v>Not irrigated</v>
       </c>
       <c r="G35" s="51">
-        <f>Common_InputFunctions.CommonCropping_GetFracWET($I$16,F35,#REF!,#REF!,Table_SourceData_FracWETIrrigation[Irrigation type i],Table_SourceData_FracWETIrrigation[FracWET])</f>
+        <f>Common_InputFunctions.CommonCropping_GetFracWET($I$16,F35,Table_SourceData_FracWET[Is in leaching zone],Table_SourceData_FracWET[FracWET],Table_SourceData_FracWETIrrigation[Irrigation type i],Table_SourceData_FracWETIrrigation[FracWET])</f>
         <v>0</v>
       </c>
     </row>
@@ -29309,7 +29309,7 @@
         <v>Not irrigated</v>
       </c>
       <c r="G36" s="51">
-        <f>Common_InputFunctions.CommonCropping_GetFracWET($I$16,F36,#REF!,#REF!,Table_SourceData_FracWETIrrigation[Irrigation type i],Table_SourceData_FracWETIrrigation[FracWET])</f>
+        <f>Common_InputFunctions.CommonCropping_GetFracWET($I$16,F36,Table_SourceData_FracWET[Is in leaching zone],Table_SourceData_FracWET[FracWET],Table_SourceData_FracWETIrrigation[Irrigation type i],Table_SourceData_FracWETIrrigation[FracWET])</f>
         <v>0</v>
       </c>
     </row>
@@ -29326,7 +29326,7 @@
         <v>Not irrigated</v>
       </c>
       <c r="G37" s="51">
-        <f>Common_InputFunctions.CommonCropping_GetFracWET($I$16,F37,#REF!,#REF!,Table_SourceData_FracWETIrrigation[Irrigation type i],Table_SourceData_FracWETIrrigation[FracWET])</f>
+        <f>Common_InputFunctions.CommonCropping_GetFracWET($I$16,F37,Table_SourceData_FracWET[Is in leaching zone],Table_SourceData_FracWET[FracWET],Table_SourceData_FracWETIrrigation[Irrigation type i],Table_SourceData_FracWETIrrigation[FracWET])</f>
         <v>0</v>
       </c>
     </row>
@@ -29343,7 +29343,7 @@
         <v>Drip irrigation</v>
       </c>
       <c r="G38" s="51">
-        <f>Common_InputFunctions.CommonCropping_GetFracWET($I$16,F38,#REF!,#REF!,Table_SourceData_FracWETIrrigation[Irrigation type i],Table_SourceData_FracWETIrrigation[FracWET])</f>
+        <f>Common_InputFunctions.CommonCropping_GetFracWET($I$16,F38,Table_SourceData_FracWET[Is in leaching zone],Table_SourceData_FracWET[FracWET],Table_SourceData_FracWETIrrigation[Irrigation type i],Table_SourceData_FracWETIrrigation[FracWET])</f>
         <v>0</v>
       </c>
     </row>
@@ -29360,7 +29360,7 @@
         <v>Sprinkler irrigation</v>
       </c>
       <c r="G39" s="51">
-        <f>Common_InputFunctions.CommonCropping_GetFracWET($I$16,F39,#REF!,#REF!,Table_SourceData_FracWETIrrigation[Irrigation type i],Table_SourceData_FracWETIrrigation[FracWET])</f>
+        <f>Common_InputFunctions.CommonCropping_GetFracWET($I$16,F39,Table_SourceData_FracWET[Is in leaching zone],Table_SourceData_FracWET[FracWET],Table_SourceData_FracWETIrrigation[Irrigation type i],Table_SourceData_FracWETIrrigation[FracWET])</f>
         <v>1</v>
       </c>
     </row>
@@ -29377,7 +29377,7 @@
         <v>Not irrigated</v>
       </c>
       <c r="G40" s="51">
-        <f>Common_InputFunctions.CommonCropping_GetFracWET($I$16,F40,#REF!,#REF!,Table_SourceData_FracWETIrrigation[Irrigation type i],Table_SourceData_FracWETIrrigation[FracWET])</f>
+        <f>Common_InputFunctions.CommonCropping_GetFracWET($I$16,F40,Table_SourceData_FracWET[Is in leaching zone],Table_SourceData_FracWET[FracWET],Table_SourceData_FracWETIrrigation[Irrigation type i],Table_SourceData_FracWETIrrigation[FracWET])</f>
         <v>0</v>
       </c>
     </row>
@@ -29394,7 +29394,7 @@
         <v>Surface irrigation</v>
       </c>
       <c r="G41" s="51">
-        <f>Common_InputFunctions.CommonCropping_GetFracWET($I$16,F41,#REF!,#REF!,Table_SourceData_FracWETIrrigation[Irrigation type i],Table_SourceData_FracWETIrrigation[FracWET])</f>
+        <f>Common_InputFunctions.CommonCropping_GetFracWET($I$16,F41,Table_SourceData_FracWET[Is in leaching zone],Table_SourceData_FracWET[FracWET],Table_SourceData_FracWETIrrigation[Irrigation type i],Table_SourceData_FracWETIrrigation[FracWET])</f>
         <v>1</v>
       </c>
     </row>
@@ -29411,7 +29411,7 @@
         <v>Not irrigated</v>
       </c>
       <c r="G42" s="51">
-        <f>Common_InputFunctions.CommonCropping_GetFracWET($I$16,F42,#REF!,#REF!,Table_SourceData_FracWETIrrigation[Irrigation type i],Table_SourceData_FracWETIrrigation[FracWET])</f>
+        <f>Common_InputFunctions.CommonCropping_GetFracWET($I$16,F42,Table_SourceData_FracWET[Is in leaching zone],Table_SourceData_FracWET[FracWET],Table_SourceData_FracWETIrrigation[Irrigation type i],Table_SourceData_FracWETIrrigation[FracWET])</f>
         <v>0</v>
       </c>
     </row>
@@ -29811,6 +29811,10 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgAFwAdQAwADAAMgA3AEYAcgB5AFwAdQAwADAAMgA3ACAAdABvACAAXAB1ADAAMAAyADcARAByAHkAXAB1ADAAMAAyADcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADIAMAAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0AGUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFQAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAUAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEUAVAAgAD0AIABwAG8AdABlAG4AdABpAGEAbAAgAGUAdgBhAHAAbwB0AHIAYQBuAHMAcABpAHIAYQB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAE0AQQBUACAAbQBpAG4AIABhAG4AZAAgAE0AQQBUACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AZQBkAGkAYQBuACAAQQBuAG4AdQBhAGwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAAoAE0AQQBUACkAXAAiACwAIABcACIATQBpAG4AIABNAEEAVABcACIALAAgAFwAIgBNAGEAeAAgAE0AQQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiIAAyADYAIABDAFwAIgAsACAAMgA2ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgAFwAIgAxADUAIAAtACAAMgA1ACAAQwBcACIALAAgADEANQAsACAAMgA1AC4AOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIiAAMQA0ACAAQwBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEANAAuADkAOQA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABaAG8AbgBlAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAXAB1ADAAMAAzAGUAIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAXAB1ADAAMAAzAGUAowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoADMALgBEAC4AYgAuADIAKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAMAAuADIANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AIAAzAC4ARAAuAEIAXwAxADAAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAGwAZQBhAGMAaABcACIALAAwAC4AMAAxADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcAG4ATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADUALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAGoAXAAiACwAXAAiAEUARgBOADIATwBcACIALAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5AFwAIgAsACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAA1ADkALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAXAAiACwAMAAuADAAMAA3ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABsAG8AdwAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAMgA5ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAOAAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAMAAuADAAMQA5ADkALAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsADAALgAwADAANQAzACwAIABcACIAQwBvAHQAdABvAG4AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAMAAuADAAMAA2ADQALAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABjAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnACkAXAAiACwAMAAuADAAMAAzACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBDAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABzAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnACkAXAAiACwAMAAuADAAMAA1ACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBTAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAMAAuADAAMAAyADYALAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABkAHUAcABsAGkAYwBhAHQAZQAgAFwAdQAwADAAMgA3AEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcAHUAMAAwADIANwAsACAAXAB1ADAAMAAyADcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcAHUAMAAwADIANwAgAGEAbgBkACAAXAB1ADAAMAAyADcAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AG4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAdQAwADAAMgA3ACAAcgBvAHcAIAB3AGkAdABoACAAcwBhAG0AZQAgAEUARgAgAGYAbwByACAAbABvAHcAIABhAG4AZAAgAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXABuAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXABuAEkAUABDAEMAOgAgAE4AMgBPACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATQBBAE4AQQBHAEUARAAgAFMATwBJAEwAUwAsACAAQQBOAEQAIABDAE8AMgAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAEwASQBNAEUAIABBAE4ARAAgAFUAUgBFAEEAIABBAFAAUABMAEkAQwBBAFQASQBPAE4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAFcARQBUACAAZgBvAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEkAUABDAEMAIAAyADAAMQA5ACAAUgBlAGYAaQBuAGUAbQBlAG4AdAAgAFYAbwBsAHUAbQBlACAANAA6ACAAQwBoAGEAcAB0AGUAcgAgADEAMQA6ACAATgAyAE8AIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAGEAbgBhAGcAZQBkACAAUwBvAGkAbABzACwAIABhAG4AZAAgAEMATwAyACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATABpAG0AZQAgAGEAbgBkACAAVQByAGUAYQAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlACAAaQByAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBwAHIAaQBuAGsAbABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAcgBmAGEAYwBlACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABUAGEAYgBsAGUAIABjAHIAZQBhAHQAZQBkACAAYgBhAHMAZQBkACAAbwBuACAAVgBFAEUAUgBHACAAdABlAHgAdAAgAFwAdQAwADAAMgA3AEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuAFwAdQAwADAAMgA3AFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAOgAgAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAFAAUgBQACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAFAAUgBQAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAB1ADAAMAAyADcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAdQAwADAAMgA3ACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AbwBuAHQAaABzACAAdABvACAAUwBlAGEAcwBvAG4AcwAgAE0AYQBwAHAAaQBuAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AbgB0AGgAXAAiACwAIABcACIAUwBlAGEAcwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAYQBuAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBiAHIAdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHIAYwBoAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHAAcgBpAGwAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQB5AFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbgBlAFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbAB5AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAZwB1AHMAdABcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAHAAdABlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AYwB0AG8AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB2AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGMAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAbgB1AHIAZQAgAE0AYQBuAGEAZwBlAG0AZQBuAHQAIAATICAATQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHAAZQByACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGkAbQApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA4AC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAyACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAIAAoALoAQwApAFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAUwBsAHUAcgByAHkAIAAoAHcAaQB0AGgAbwB1AHQAIABuAGEAdAB1AHIAYQBsACAAYwByAHUAcwB0ACkAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAGIAKQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABTAHQAbwByAGEAZwBlACAAXAB1ADAAMAAzAGMAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AFAAbwB1AGwAdAByAHkAIAB3AGkAdABoACAAYQBuAGQAIAB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABzAGUAcABhAHIAYQB0AGUAIABOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE0AQQBUACAAcgBhAHcAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAbABsAG8AdwAgAGwAbwBvAGsAdQBwACAAbwBmACAAbgB1AG0AYgBlAHIAcwAuAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBuAGQAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAcgBlAHQAdQByAG4AZQBkACAAdABvACAAdABoAGUAIABzAG8AaQBsAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AaQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADEALgA0AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBOAGkAIABcAHUAMAAwADIANgAgAEUARgBOADIATwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAE4AMgBPACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUATgAyAE8AOgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXABuAEcAVwBQAE4AMgBPADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBOADIATwAsACAARwBXAFAAXwBOADIATwAsAFwAbgAgACAAIAAgAEUAXwBOADIATwAgACoAIABHAFcAUABfAE4AMgBPAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAE4AMgBPACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AE4AMgBPAH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AE4AMgBPAH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBOADIATwBcACIALABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAATgAyAE8AXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAEMASAA0ACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUAQwBIADQAOgAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXABuAEcAVwBQAEMASAA0ADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBDAEgANAAsACAARwBXAFAAXwBDAEgANAAsAFwAbgAgACAAIAAgAEUAXwBDAEgANAAgACoAIABHAFcAUABfAEMASAA0AFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEMASAA0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AEMASAA0AH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AEMASAA0AH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBDAEgANABcACIALABcACIATQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAAQwBIADQAXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAbABpAHYAZQBzAHQAbwBjAGsAIAB0AHkAcABlAHMAXABuAEUAeABjAGUAbAAgAG0AbwBkAHUAbABlACAAbgBhAG0AZQA6ACAAUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBcAG4ARgByAGEAYwBXAEUAVABNAE0AUwBpACAAPQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4AKABUAGEAYgBsAGUAIABBADUALgA1AC4AMQAwAC4AMgAgAGkAcwAgAHIAZQBmAGUAcgBlAG4AYwBlAGQAIABpAG4AIABOAEkAUgAgAGIAdQB0ACAAMQAgAGkAcwAgAHUAcwBlAGQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAxACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXABuAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTACAAPQAgADAALgAwADIAIAAoAEcAZwAgAE4ALwBHAGcAIABhAHAAcABsAGkAZQBkACkAIAAoAEMAUwAgAEUARgAsACAAcwBvAHUAcgBjAGUAIABJAFAAQwBDACAAKAAyADAAMQA5ACkAKQAgAFwAbgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAbABvAHMAdAAgAHQAaAByAG8AdQBnAGgAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAIAAwAC4AMAAwADUAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsACAAMAAuADAAMAA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAgADAALgAwADAAMQA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcABcACIALAAgADAALgAwADAANAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAIABjAGEAbgBlAFwAIgAsACAAMAAuADAAMQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAMAAuADAAMAA1ADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAMAAuADAAMAA2ADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXABuAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVgBhAGkAcgBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE0AUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAAVABhAGIAbABlACAANQAuADEAMgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAOQAsACAAMwAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AG0AYgBvAGwAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgAgACgAbQA9ADEAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADIAXAAiACwAIABcACIATABpAHEAdQBpAGQAIABzAHkAcwB0AGUAbQBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwAgACgAbQA9ADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAG0APQAzACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGEAXAAiACwAIABcACIAUwB1AG0AcAAgAGEAbgBkACAAZABpAHMAcABlAHIAcwBhAGwAIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtACAAKABtAD0AMwBhACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGIAXAAiACwAIABcACIARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAEQAcgBhAGkAbgBzACAAdABvACAAcABhAGQAZABvAGMAawAgACgAbQA9ADMAYgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIANABcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAIAAoAG0APQA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA1AFwAIgAsACAAXAAiAEQAcgB5AGwAbwB0ACAAKABmAGUAZQBkACAAcABhAGQAKQBcACIALAAgAFwAIgBEAHIAeQBsAG8AdAAgACgAZgBlAGUAZAAgAHAAYQBkACkAIAAoAG0APQA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA2AFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQAgACgAbQA9ADYAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADcAXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwAgACgAbQA9ADcAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADgAXAAiACwAIABcACIARABlAGUAcAAgAGwAaQB0AHQAZQByAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgAgACgAbQA9ADgAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADkAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQAgACgAbQA9ADkAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMABcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwAgACgAbQA9ADEAMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnACAAKABtAD0AMQAxACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADEAYQBcACIALAAgAFwAIgBCAGUAbAB0ACAAbQBhAG4AdQByAGUAIAByAGUAbQBvAHYAYQBsAFwAIgAsACAAXAAiAEIAZQBsAHQAIABtAGEAbgB1AHIAZQAgAHIAZQBtAG8AdgBhAGwAIAAoAG0APQAxADEAYQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAGIAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABzAHQAbwByAGUAZAAgAGkAbgAgAGgAbwB1AHMAZQBcACIALAAgAFwAIgBNAGEAbgB1AHIAZQAgAHMAdABvAHIAZQBkACAAaQBuACAAaABvAHUAcwBlACAAKABtAD0AMQAxAGIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAKABtAD0AMQAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADMAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAG0APQAxADMAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEANABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAIAAoAG0APQAxADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQgBlAGUAZgAgAGMAYQB0AHQAbABlACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAYQB0AHQAbABlACwAIABmAG8AcgAgAG0AYQBuAHUAZgBhAGMAdAB1AHIAaQBuAGcAIABiAGUAZQBmAFwAIgAsACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBhAHQAdABsAGUALAAgAGYAbwByACAAcAByAGkAbQBlACAAYgBlAGUAZgBcACIALAAgAFwAIgBOAFMAVwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAYQB0AHQAbABlACwAIAB3AGUAYQBuAGUAcgBzAFwAIgAsACAAXAAiAE4AVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFEATABEAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAVABBAFMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBWAEkAQwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFcAQQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBDAGgAaQBjAGsAZQBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEMAaABpAGMAawBlAG4AcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBoAGkAYwBrAGUAbgBzACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQwBoAGkAYwBrAGUAbgBzAF8AVgBhAGkAcgBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEMAaABpAGMAawBlAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQwBoAGkAYwBrAGUAbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBDAGgAaQBjAGsAZQBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAG8AZAB1AGMAdABcACIALAAgAFwAIgBTAG8AdQByAGMAZQAgAHIAZQBnAGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBoAGkAYwBrAGUAbgBzAFwAIgAsACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEQAYQBpAHIAeQBjAGEAdAB0AGwAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABwAHIAbwBkAHUAYwB0AHMAIABmAG8AcgAgAHMAYwBvAHAAZQAgADMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXwBWAGEAaQByAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8ARABhAGkAcgB5AGMAYQB0AHQAbABlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATABpAGYAZQBjAHkAYwBsAGUAcwAuACAAKAAyADAAMgA2ACkALgAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABHAGEAcwAgAEUAbQBpAHMAcwBpAG8AbgAgAEkAbgB0AGUAbgBzAGkAdABpAGUAcwAgAGYAbwByACAATQBhAHQAZQByAGkAYQBsACAASQBuAHAAdQB0AHMAIAB0AG8AIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAQQBnAHIAaQBjAHUAbAB0AHUAcgBlACwAIABGAGkAcwBoAGUAcgBpAGUAcwAgAGEAbgBkACAARgBvAHIAZQBzAHQAcgB5AC4AIABWAGUAcgBzAGkAbwBuACAANAA4AC4AIABkAG8AaQAgADEAMAAuADUAMgA4ADEALwB6AGUAbgBvAGQAbwAuADEAOQA2ADUANgA1ADgAMABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEQAYQBpAHIAeQBjAGEAdAB0AGwAZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AFwAIgAsACAAXAAiAFMAbwB1AHIAYwBlACAAcgBlAGcAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAaQByAHkAIABjAG8AdwBzAFwAIgAsACAAXAAiAFYASQBDAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBQAGkAZwBzACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUABpAGcAcwBfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAaQBnAHMAXAAiACwAIABcACIAQQB1AHMAdAByAGEAbABpAGEAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUwBoAGUAZQBwAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBTAGgAZQBlAHAAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFMAaABlAGUAcAAgAHAAcgBvAGQAdQBjAHQAcwAgAGYAbwByACAAcwBjAG8AcABlACAAMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFMAaABlAGUAcABfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBTAGgAZQBlAHAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFMAaABlAGUAcABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBMAGkAZgBlAGMAeQBjAGwAZQBzAC4AIAAoADIAMAAyADYAKQAuACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAEcAYQBzACAARQBtAGkAcwBzAGkAbwBuACAASQBuAHQAZQBuAHMAaQB0AGkAZQBzACAAZgBvAHIAIABNAGEAdABlAHIAaQBhAGwAIABJAG4AcAB1AHQAcwAgAHQAbwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABBAGcAcgBpAGMAdQBsAHQAdQByAGUALAAgAEYAaQBzAGgAZQByAGkAZQBzACAAYQBuAGQAIABGAG8AcgBlAHMAdAByAHkALgAgAFYAZQByAHMAaQBvAG4AIAA0ADgALgAgAGQAbwBpACAAMQAwAC4ANQAyADgAMQAvAHoAZQBuAG8AZABvAC4AMQA5ADYANQA2ADUAOAAwAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUwBoAGUAZQBwAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAaABlAGUAcAAsACAAZgBvAHIAIABtAHUAdAB0AG8AbgBcACIALAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAaABlAGUAcAAsACAAZgBvAHIAIABwAHIAaQBtAGUAIABsAGEAbQBiAFwAIgAsACAAXAAiAE4AUwBXAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAUQBMAEQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBTAEEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFYASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAVwBBAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFIATwBXACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwAKQAgACsAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACAALQAgADEAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAVABhAGIAbABlAEgAZQBhAGQAZQByAEMAZQBsAGwALABcAG4AIAAgAEMATwBMAFUATQBOACgAVABhAGIAbABlAEgAZQBhAGQAZQByAEMAZQBsAGwAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAHIAYQB5AEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIABBAHIAcgBhAHkARABhAHQAYQAsACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkALAAgAFsAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQBdACwAXABuACAASQBGAEUAUgBSAE8AUgAoAFwAbgAgACAAIAAgACAASQBOAEQARQBYACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFUATgBJAFEAVQBFACgAQQByAHIAYQB5AEQAYQB0AGEAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBXACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABDAE8ATABVAE0ATgAoACkALQBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5ACkALAAgADEALAAgAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALAAgAFwAIgBcACIAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABJAEYAKABJAFMATgBVAE0AQgBFAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkAXABuACAAIAAgACAAKQAsACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQAsACAAMAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAVAB3AG8AQwBvAGwAdQBtAG4AcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIAAoAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlADEAKQAqACgATABvAG8AawB1AHAAQQByAHIAYQB5ADIAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgApACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAKQAsACAAXAAiAFwAIgAsACAAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAKQApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABbAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlAF0ALABcAG4AIAAgACAAIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBmAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBmAEYAYQBsAHMAZQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABDAGUAbABsACwAIABEAGUAbABpAG0AaQB0AGUAcgAsACAAWwBDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQBdACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyAF0ALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSAFgATQBMACgAXABuACAAIAAgACAAIAAgACAAIABcACIAXAB1ADAAMAAzAGMAdABcAHUAMAAwADMAZQBcAHUAMAAwADMAYwBzAFwAdQAwADAAMwBlAFwAIgAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAUwBVAEIAUwBUAEkAVABVAFQARQAoAEMAZQBsAGwALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQAsAFwAIgBcACIAKQAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAZQBsAGkAbQBpAHQAZQByACwAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwBzAFwAdQAwADAAMwBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgACkAIABcAHUAMAAwADIANgBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwAvAHMAXAB1ADAAMAAzAGUAXAB1ADAAMAAzAGMALwB0AFwAdQAwADAAMwBlAFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAC8ALwBzAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAYQB2AGcAVABlAG0AcAAsAGEAdgBnAFIAYQBpAG4ALABmAHIAbwBzAHQARABhAHkAcwAsAGUAbABlAHYALABtAGEAcABfAHAAZQB0ACwAXABuACAAIAAgACAAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkALABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQAsAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABtAGEAeABFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBQAEUAVABBAHIAcgBhAHkALABtAGEAeABQAEUAVABBAHIAcgBhAHkALABcAG4AIAAgACAAIABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBSAGEAaQBuACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AZgByAG8AcwB0AEQAYQB5AHMAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABGAHIAbwBzAHQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AZQBsAGUAdgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AZQBsAGUAdgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAFAARQBUAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AbQBhAHAAXwBwAGUAdAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFAARQBUAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AbQBhAHAAXwBwAGUAdAApACwAXABuACAAIAAgACAAIAAgACAAIABUAEEASwBFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgAYwBsAGkAbQBhAHQAZQBaAG8AbgBlAEEAcgByAGEAeQAsAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAMQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATQBpAG4AQQByAHIAYQB5ACwAIABNAGEAeABBAHIAcgBhAHkALAAgAEkAdABlAG0AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBpAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGEAeABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACwAXABuACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAEkAdABlAG0AQQByAHIAYQB5ACwAIABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABDAHIAaQB0AGUAcgBpAGEAMQAsACAAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkALAAgAFEAdQBhAG4AdABpAHQAeQAsACAAWwBNAHUAbAB0AGkAcABsAGkAZQByAF0ALAAgAFsAQwByAGkAdABlAHIAaQBhADIAXQAsAFsAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AF0ALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAbQB1AGwAdABpAHAAbABpAGUAcgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABNAHUAbAB0AGkAcABsAGkAZQByACkALAAxACwATQB1AGwAdABpAHAAbABpAGUAcgApACwAXABuACAAIAAgACAAcQB1AGEAbgB0AGkAdAB5ACwAIABRAHUAYQBuAHQAaQB0AHkAKgBNAHUAbAB0AGkAcABsAGkAZQByACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAxACkALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMgAsAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwByAGkAdABlAHIAaQBhADIAKQAsADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMgApACkALABcAG4AIAAgACAAIABTAFUATQBQAFIATwBEAFUAQwBUACgAYwByAGkAdABlAHIAaQBhADEAKgBjAHIAaQB0AGUAcgBpAGEAMgAqAHEAdQBhAG4AdABpAHQAeQApAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAXAB1ADAAMAAzAGMAIABTACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAXAB1ADAAMAAzAGUAIABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAIAAvACoAaABlAGwAcABlAHIAOgAgAGUAbgBkACAAZABhAHQAZQAgAGYAbwByACAAYQAgAHIAZQBwAG8AcgB0AGkAbgBnACAAcABlAHIAaQBvAGQAIABzAHQAYQByAHQAaQBuAGcAIABhAHQAIABhACAAZwBpAHYAZQBuACAAZABhAHQAZQAqAC8AXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALAAgAC8AKgBvAG4AbAB5ACAAbgBlAGUAZAAgAHQAbwAgAGwAbwBvAGsAIABiAGEAYwBrACAAMwA2ADUAIABkAGEAeQBzACgAbQBhAHgAIABvAHYAZQByAGwAYQBwACAAdwBpAG4AZABvAHcAKQAqAC8AXABuACAAIAAgACAAIAAgACAAIABBACwAUwAtADMANgA1ACwAXABuACAAIAAgACAAIAAgACAAIAB5AGEALABZAEUAQQBSACgAQQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AGIALABZAEUAQQBSACgARQApACwAIAAvACoAaQBmACAAdABoAGUAIABhAG4AYwBoAG8AcgAgAGYAbwByACAAeQBhACAAZQBuAGQAcwAgAGIAZQBmAG8AcgBlACAAUwAsAGkAdAAgAGMAYQBuAFwAdQAwADAAMgA3AHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAbgBlAHgAdAAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQBcAHUAMAAwADMAYwBTACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGIAIABzAHQAYQByAHQAcwAgAGEAZgB0AGUAcgAgAEUALABpAHQAIABjAGEAbgBcAHUAMAAwADIANwB0ACAAbwB2AGUAcgBsAGEAcAA7ACAAbQBvAHYAZQAgAHQAbwAgAHAAcgBlAHYAaQBvAHUAcwAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQBcAHUAMAAwADMAZQBFACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4ALABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQByAHMALABTAEUAUQBVAEUATgBDAEUAKABuACwAMQAsAGYAaQByAHMAdABZAGUAYQByACwAMQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwAsAEQAQQBUAEUAKAB5AHIAcwAsAG0ALABkACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMALABNAEEAUAAoAHMAdABhAHIAdABzACwAUABlAHIAaQBvAGQARQBuAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAdABhAGcALABJAEYAKABzAHQAYQByAHQAcwA9AFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcACIAIAAoAFQAaABpAHMAIAByAGUAcABvAHIAdABpAG4AZwAgAGMAeQBjAGwAZQApAFwAIgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMAVABlAHgAdAAsAFQARQBYAFQAKABzAHQAYQByAHQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMAVABlAHgAdAAsAFQARQBYAFQAKABlAG4AZABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbgA9ADAALABcACIAXAAiACwASABTAFQAQQBDAEsAKABzAHQAYQByAHQAcwBUAGUAeAB0ACAAXAB1ADAAMAAyADYAIABcACIAIAB0AG8AIABcACIAIABcAHUAMAAwADIANgAgAGUAbgBkAHMAVABlAHgAdAAgAFwAdQAwADAAMgA2ACAAdABhAGcAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlAFwAbgA9AEwAQQBNAEIARABBACgARgB1AG4AYwB0AGkAbwBuACwAIABUAEUAWABUAEIARQBGAE8AUgBFACgARgBPAFIATQBVAEwAQQBUAEUAWABUACgARgB1AG4AYwB0AGkAbwBuACkALAAgAFwAIgAoAFwAIgApACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQAsAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAD0AXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAIAA9ACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgAMQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkAPQBQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQA9AEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQA9AFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAXAB1ADAAMAAzAGUAMAAsACAAMQAsACAAMAApAFwAbgAgACAAIAAgACkAKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBDAG8AbgB2AGUAcgB0AFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAFQAbwBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlACwAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAQQByAHIAYQB5ACwAIABTAHQAYQB0AGUAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlACwAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAFwAbgA9AEwAQQBNAEIARABBACgAVABhAHIAZwBlAHQAQwBlAGwAbAAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABzAGgALAAgAFQARQBYAFQAQQBGAFQARQBSACgAQwBFAEwATAAoAFwAIgBmAGkAbABlAG4AYQBtAGUAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALAAgAFwAIgBdAFwAIgApACwAXABuACAAIAAgACAAYQBkAGQAcgAsACAAQwBFAEwATAAoAFwAIgBhAGQAZAByAGUAcwBzAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAXABuACAAIAAgACAAXAAiACMAXAB1ADAAMAAyADcAXAAiACAAXAB1ADAAMAAyADYAIABzAGgAIABcAHUAMAAwADIANgAgAFwAIgBcAHUAMAAwADIANwAhAFwAIgAgAFwAdQAwADAAMgA2ACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBEAGkAZgBmAGUAcgBlAG4AdABTAGgAZQBlAHQAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcACIAIABcAHUAMAAwADIANgAgAGEAZABkAHIAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADEAXwAyAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAXABuACAAIAAgACAAQwBIAE8ATwBTAEUAQwBPAEwAUwAoAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsACAAMQAsACAAMgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADMAXwA0AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAXABuACAAIAAgACAAQwBIAE8ATwBTAEUAQwBPAEwAUwAoAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsACAAMwAsACAANAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEcAZQB0AE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACwAIABNAE0AUwAsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAXABuACAAIAAgACAAIAAgACAAIABNAEUARABJAEEATgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAE8AVQBOAEQAKABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgADAAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0ASQBOACgAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBBAFgAKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATQBNAFMALAAgAE0ATQBTAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBSAGUAcwB1AGwAdABzAEkAdABlAG0ARgByAG8AbQBFAHEAdQBhAHQAaQBvAG4AVABpAHQAbABlAEEAbgBkAFMAbwB1AHIAYwBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABpAHQAbABlAEMAZQBsAGwALAAgAFMAbwB1AHIAYwBlAEMAZQBsAGwALABcAG4AIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgATABFAEYAVAAoAFMAbwB1AHIAYwBlAEMAZQBsAGwALAAgAEYASQBOAEQAKABcACIALABcACIALAAgAFMAbwB1AHIAYwBlAEMAZQBsAGwAKQAgAC0AMQApACwAIABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAXAAiACwAIABcACIAXAAiACkAIABcAHUAMAAwADIANgAgAFwAIgAgAFwAIgAgAFwAdQAwADAAMgA2ACAAVABpAHQAbABlAEMAZQBsAGwAXABuACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAXAB1ADAAMAAzAGUAMAAsACAAMQAsACAAMAApAFwAbgAgACAAIAAgACkAKQA7AFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEMAYQBsAGMAdQBsAGEAdABlAEgAYQByAHYAZQBzAHQASQBuAGQAZQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQwByAG8AcABUAHkAcABlACwAIABDAHIAbwBwAFQAeQBwAGUAQQByAHIAYQB5ACwAIABSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgADEALwAoADEAKwBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAEMAcgBvAHAAVAB5AHAAZQAsACAAQwByAG8AcABUAHkAcABlAEEAcgByAGEAeQAsACAAUgBlAHMAaQBkAHUAZQBDAHIAbwBwAFIAYQB0AGkAbwBBAHIAcgBhAHkAKQApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAASABhAHIAdgBlAHMAdABJAG4AZABlAHgALABcAG4AIAAgACAAIAAoADEALQBIAGEAcgB2AGUAcwB0AEkAbgBkAGUAeAApAC8ASABhAHIAdgBlAHMAdABJAG4AZABlAHgAXABuACkAOwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBGAHIAYQBjAHQAaQBvAG4AUgBlAHMAaQBkAHUAZQBSAGUAbQBvAHYAZQBkAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABvAHQAYQBsAFIAZQBzAGkAZAB1AGUALAAgAEEAbQBvAHUAbgB0AFIAZQBtAG8AdgBlAGQALABcAG4AIAAgACAAIAAoAEEAbQBvAHUAbgB0AFIAZQBtAG8AdgBlAGQAKgAxADAAXgAzACkALwAoAFQAbwB0AGEAbABSAGUAcwBpAGQAdQBlACoAMQAwAF4AMwApAFwAbgApACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4ANQAuADEAOgAgAE8AdABoAGUAcgAgAEwAaQB2AGUAcwB0AG8AYwBrACAALQAgAEUAbgB0AGUAcgBpAGMAIABmAGUAcgBtAGUAbgB0AGEAdABpAG8AbgAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABlAGEAYwBoACAAbwB0AGgAZQByACAAbABpAHYAZQBzAHQAbwBjAGsAIAB0AHkAcABlACAAKABrAGcAIABDAEgANAAvAGgAZQBhAGQALwB5AGUAYQByACkAIAAoAE0AagApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATwB0AGgAZQByACAATABpAHYAZQBzAHQAbwBjAGsAIAAtACAARQBuAHQAZQByAGkAYwAgAGYAZQByAG0AZQBuAHQAYQB0AGkAbwBuACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGUAYQBjAGgAIABvAHQAaABlAHIAIABsAGkAdgBlAHMAdABvAGMAawAgAHQAeQBwAGUAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBqAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABDAEgANAAgAC8AIABoAGUAYQBkACAALwAgAHkAZQBhAHIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADUALgAxAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAyACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AdABoAGUAcgAgAEwAaQB2AGUAcwB0AG8AYwBrACAAVAB5AHAAZQBcACIALAAgAFwAIgBNAGoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBmAGYAYQBsAG8AXAAiACwAIAA2ADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBvAGEAdABzAFwAIgAsACAANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGUAZQByAFwAIgAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAYQBtAGUAbABzAFwAIgAsACAANAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbABwAGEAYwBhAHMAXAAiACwAIAA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHMAZQBzAFwAIgAsACAAMQA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AdQBsAGUAcwAvAGEAcwBzAGUAcwBcACIALAAgADEAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AdQBzAC8AbwBzAHQAcgBpAGMAaABlAHMAXAAiACwAIAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBQAHIAbwBkAHUAYwBlAGQAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4ANQAuADIAOgAgAE8AdABoAGUAcgAgAEwAaQB2AGUAcwB0AG8AYwBrACAALQAgAFYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZABzACAAcAByAG8AZAB1AGMAZQBkACAAYgB5ACAAZQBhAGMAaAAgAG8AdABoAGUAcgAgAGwAaQB2AGUAcwB0AG8AYwBrACAAdAB5AHAAZQAgACgAawBnACAAVgBTAC8AaABlAGEAZAAvAGQAYQB5ACkAIAAoAFYAUwBqACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBQAHIAbwBkAHUAYwBlAGQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE8AdABoAGUAcgAgAEwAaQB2AGUAcwB0AG8AYwBrACAALQAgAFYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZABzACAAcAByAG8AZAB1AGMAZQBkACAAYgB5ACAAZQBhAGMAaAAgAG8AdABoAGUAcgAgAGwAaQB2AGUAcwB0AG8AYwBrACAAdAB5AHAAZQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBQAHIAbwBkAHUAYwBlAGQAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAUwBqAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFAAcgBvAGQAdQBjAGUAZABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAFYAUwAgAC8AIABoAGUAYQBkACAALwAgAGQAYQB5AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFAAcgBvAGQAdQBjAGUAZABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADUALgAyAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFAAcgBvAGQAdQBjAGUAZABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBQAHIAbwBkAHUAYwBlAGQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOQAsACAAMgAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAHQAaABlAHIAIABMAGkAdgBlAHMAdABvAGMAawAgAFQAeQBwAGUAXAAiACwAIABcACIAVgBTAGoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBmAGYAYQBsAG8AXAAiACwAIAAyAC4ANwAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAbwBhAHQAcwBcACIALAAgADAALgAzADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGUAcgBcACIALAAgADAALgA5ADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBhAG0AZQBsAHMAXAAiACwAIAAyAC4ANwAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbABwAGEAYwBhAHMAXAAiACwAIAAwAC4AMwA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHMAZQBzAFwAIgAsACAAMgAuADcAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAHUAbABlAHMALwBhAHMAcwBlAHMAXAAiACwAIAAwAC4AOQAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAbQB1AHMALwBvAHMAdAByAGkAYwBoAGUAcwBcACIALAAgADAALgAzADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGUAZABcAG4AVABhAGIAbABlACAAQQAuADEALgA1AC4AMwA6ACAATwB0AGgAZQByACAATABpAHYAZQBzAHQAbwBjAGsAIAAtACAATgBpAHQAcgBvAGcAZQBuACAAZQB4AGMAcgBlAHQAZQBkACAAcABlAHIAIABsAGkAdgBlAHMAdABvAGMAawAgAHQAeQBwAGUAIAAoAGsAZwAgAE4AMgBPAC8AaABlAGEAZAAvAHkAZQBhAHIAKQAgACgATgBFAGoAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGUAZABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATwB0AGgAZQByACAATABpAHYAZQBzAHQAbwBjAGsAIAAtACAATgBpAHQAcgBvAGcAZQBuACAAZQB4AGMAcgBlAHQAZQBkACAAcABlAHIAIABsAGkAdgBlAHMAdABvAGMAawAgAHQAeQBwAGUAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAZQBkAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAEUAagBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABlAGQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAgAC8AIABoAGUAYQBkACAALwAgAHkAZQBhAHIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAZQBkAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4ANQAuADMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAZQBkAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGUAZABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAyACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AdABoAGUAcgAgAEwAaQB2AGUAcwB0AG8AYwBrACAAVAB5AHAAZQBcACIALAAgAFwAIgBOAEUAagBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgB1AGYAZgBhAGwAbwBcACIALAAgADMAOQAuADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBvAGEAdABzAFwAIgAsACAANwAuADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGUAcgBcACIALAAgADEAMwAuADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBhAG0AZQBsAHMAXAAiACwAIAAzADkALgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbABwAGEAYwBhAHMAXAAiACwAIAA3AC4AMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAG8AcgBzAGUAcwBcACIALAAgADMAOQAuADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQB1AGwAZQBzAC8AYQBzAHMAZQBzAFwAIgAsACAAMQAzAC4AMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AdQBzAC8AbwBzAHQAcgBpAGMAaABlAHMAXAAiACwAIAA3AC4AMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBBAHYAZQByAGEAZwBlAEwAaQB2AGUAdwBlAGkAZwBoAHQAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4ANQAuADQAOgAgAE8AdABoAGUAcgAgAEwAaQB2AGUAcwB0AG8AYwBrACAALQAgAEEAdgBlAHIAYQBnAGUAIABMAGkAdgBlAHcAZQBpAGcAaAB0AHMAIAAoAFcAYwBvACkAIAAoAGsAZwApACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAEEAdgBlAHIAYQBnAGUATABpAHYAZQB3AGUAaQBnAGgAdABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATwB0AGgAZQByACAATABpAHYAZQBzAHQAbwBjAGsAIAAtACAAQQB2AGUAcgBhAGcAZQAgAEwAaQB2AGUAdwBlAGkAZwBoAHQAcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAEEAdgBlAHIAYQBnAGUATABpAHYAZQB3AGUAaQBnAGgAdABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVwBjAG8AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBBAHYAZQByAGEAZwBlAEwAaQB2AGUAdwBlAGkAZwBoAHQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBBAHYAZQByAGEAZwBlAEwAaQB2AGUAdwBlAGkAZwBoAHQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA1AC4ANABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAEEAdgBlAHIAYQBnAGUATABpAHYAZQB3AGUAaQBnAGgAdABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAEEAdgBlAHIAYQBnAGUATABpAHYAZQB3AGUAaQBnAGgAdABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADEALAAgADMALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAATABpAHYAZQBzAHQAbwBjAGsAIABUAHkAcABlACAAagBcACIALAAgAFwAIgBBAHYAZQByAGEAZwBlACAATABpAHYAZQB3AGUAaQBnAGgAdABcACIALAAgAFwAIgBBAHYAZQByAGEAZwBlACAATABpAHYAZQB3AGUAaQBnAGgAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgB1AGYAZgBhAGwAbwBcACIALAAgADMAMwA2ACwAIABcACIALQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBvAGEAdABzAFwAIgAsACAAMwAzACwAIABcACIAMgA4AGsAZwAgAC0AIABsAG8AdwAgAHAAcgBvAGQAdQBjAHQAaQB2AGkAdAB5ACAAcwB5AHMAdABlAG0AcwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBvAGEAdABzAFwAIgAsACAAMwAzACwAIABcACIANQAwAGsAZwAgAC0AIABoAGkAZwBoACAAcAByAG8AZAB1AGMAdABpAHYAaQB0AHkAIABzAHkAcwB0AGUAbQBzAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGUAZQByAFwAIgAsACAAMQAyADAALAAgADEAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAYQBtAGUAbABzAFwAIgAsACAAMgAxADcALAAgADUANwAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbABwAGEAYwBhAHMAXAAiACwAIABcACIALQBcACIALAAgADYANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAG8AcgBzAGUAcwBcACIALAAgADMANwA3ACwAIAA1ADUAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAHUAbABlAHMALwBhAHMAcwBlAHMAXAAiACwAIAAxADMAMAAsACAAMgA0ADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBtAHUAcwAvAG8AcwB0AHIAaQBjAGgAZQBzAFwAIgAsACAAMQAyADAALAAgADEAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBmAGUAcgBlAG4AYwBlAFwAIgAsACAAXAAiAEkAUABDAEMAIAAyADAAMQA5ACAAVABhAGIAbABlACAAMQAwAEEALgA1ACAAWwAyAF0AXAAiACwAIABcACIASQBQAEMAQwAgADIAMAAxADkAIABUAGEAYgBsAGUAIAAxADAALgAxADAAIABbADIAXQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ARgByAGEAYwB0AGkAbwBuAFcAYQBzAHQAZQBJAG4ATQBNAFMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4ANQAuADUAOgAgAE8AdABoAGUAcgAgAEwAaQB2AGUAcwB0AG8AYwBrACAALQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAHcAYQBzAHQAZQAgAGkAbgAgAGUAYQBjAGgAIABtAGEAbgB1AHIAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABzAHkAcwB0AGUAbQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0ATQBTAG0AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ARgByAGEAYwB0AGkAbwBuAFcAYQBzAHQAZQBJAG4ATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE8AdABoAGUAcgAgAEwAaQB2AGUAcwB0AG8AYwBrACAALQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAHcAYQBzAHQAZQAgAGkAbgAgAGUAYQBjAGgAIABtAGEAbgB1AHIAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABzAHkAcwB0AGUAbQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAEYAcgBhAGMAdABpAG8AbgBXAGEAcwB0AGUASQBuAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE0AUwBtAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ARgByAGEAYwB0AGkAbwBuAFcAYQBzAHQAZQBJAG4ATQBNAFMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBGAHIAYQBjAHQAaQBvAG4AVwBhAHMAdABlAEkAbgBNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADUALgA1AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ARgByAGEAYwB0AGkAbwBuAFcAYQBzAHQAZQBJAG4ATQBNAFMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBGAHIAYQBjAHQAaQBvAG4AVwBhAHMAdABlAEkAbgBNAE0AUwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAzACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQBcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBDAFQAXAAiACwAIAAgADkAOQAuADYANgAsACAAIAAwAC4AMwA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AUwBXAFwAIgAsACAAIAA5ADkALgA2ADYALAAgACAAMAAuADMANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAFQAXAAiACwAIAAgADkAOQAuADYANgAsACAAIAAwAC4AMwA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEATABEAFwAIgAsACAAIAA5ADkALgA2ADYALAAgACAAMAAuADMANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAEEAXAAiACwAIAAgADkAOQAuADYANgAsACAAIAAwAC4AMwA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAQQBTAFwAIgAsACAAIAA5ADkALgA2ADYALAAgACAAMAAuADMANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEkAQwBcACIALAAgACAAOQA5AC4ANgA2ACwAIAAgADAALgAzADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBBAFwAIgAsACAAIAA5ADkALgA2ADYALAAgACAAMAAuADMANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAEMAbwBuAHYAZQByAHMAaQBvAG4ARgBhAGMAdABvAHIAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4ANQAuADYAOgAgAE8AdABoAGUAcgAgAEwAaQB2AGUAcwB0AG8AYwBrACAALQAgAE0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABwAGUAcgAgAHIAZQBnAGkAbwBuACAAKABmAHIAYQBjAHQAaQBvAG4AKQAgACgATQBDAEYAaQBtACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAE0AZQB0AGgAYQBuAGUAQwBvAG4AdgBlAHIAcwBpAG8AbgBGAGEAYwB0AG8AcgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATwB0AGgAZQByACAATABpAHYAZQBzAHQAbwBjAGsAIAAtACAATQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHAAZQByACAAcgBlAGcAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAEMAbwBuAHYAZQByAHMAaQBvAG4ARgBhAGMAdABvAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AQwBGAGkAbQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAE0AZQB0AGgAYQBuAGUAQwBvAG4AdgBlAHIAcwBpAG8AbgBGAGEAYwB0AG8AcgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAE0AZQB0AGgAYQBuAGUAQwBvAG4AdgBlAHIAcwBpAG8AbgBGAGEAYwB0AG8AcgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADUALgA2AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATQBlAHQAaABhAG4AZQBDAG8AbgB2AGUAcgBzAGkAbwBuAEYAYQBjAHQAbwByAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATQBlAHQAaABhAG4AZQBDAG8AbgB2AGUAcgBzAGkAbwBuAEYAYQBjAHQAbwByAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB0AGEAdABlAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiACwAIABcACIAVQBuAGMAbwB2AGUAcgBlAGQAIABBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAEMAVABcACIALAAgACAAMAAuADAAMAA0ADcALAAgACAAMAAuADcAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAFMAVwBcACIALAAgACAAMAAuADAAMAA0ADcALAAgACAAMAAuADcANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAFQAXAAiACwAIAAgADAALgAwADAANAA3ACwAIAAgADAALgA4ADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUQBMAEQAXAAiACwAIAAgADAALgAwADAANAA3ACwAIAAgADAALgA3ADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBAFwAIgAsACAAIAAwAC4AMAAwADQANwAsACAAIAAwAC4ANwA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAQQBTAFwAIgAsACAAIAAwAC4AMAAwADQANwAsACAAIAAwAC4ANwAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYASQBDAFwAIgAsACAAIAAwAC4AMAAwADQANwAsACAAIAAwAC4ANwA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAQQBcACIALAAgACAAMAAuADAAMAA0ADcALAAgACAAMAAuADcANgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADUALgBYADoAIABPAHQAaABlAHIAIABMAGkAdgBlAHMAdABvAGMAawAgAC0AIABNAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIABwAG8AdABlAG4AdABpAGEAbAAgACgAbQAzACAAQwBIADQAIAAvACAAawBnACAAVgBTACkAIAAoAEIATwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBPAHQAaABlAHIAIABMAGkAdgBlAHMAdABvAGMAawAgAC0AIABNAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIABwAG8AdABlAG4AdABpAGEAbABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEIATwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBtADMAIABDAEgANAAgAC8AIABrAGcAIABWAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4ANQAuAFgAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBOACAAUwBPAFUAUgBDAEUAOgAgAFQAaABlAHIAZQAgAHcAZQByAGUAIABuAG8AIAB2AGEAbAB1AGUAcwAgAGkAbgAgAFYARQBFAFIARwAgAHMAbwAgAHQAaABpAHMAIABkAGEAdABhACAAaABhAHMAIABiAGUAZQBuACAAZwBlAG4AZQByAGEAdABlAGQAIABiAHkAIAB1AHMAaQBuAGcAIABkAG8AYwB1AG0AZQBuAHQAZQBkACAAQgBPACAAdgBhAGwAdQBlAHMAIABmAHIAbwBtACAAbwB0AGgAZQByACAAbABpAHYAZQBzAHQAbwBjAGsAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAATABpAHYAZQBzAHQAbwBjAGsAIABUAHkAcABlAFwAIgAsACAAXAAiAEIATwBcACIALAAgAFwAIgBUAGEAawBlAG4AIABmAHIAbwBtAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAHUAZgBmAGEAbABvAFwAIgAsACAAMAAuADEAOQAsACAAXAAiAEYAZQBlAGQAbABvAHQALAAgAFAAYQBzAHQAdQByAGUAIABiAGUAZQBmAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAG8AYQB0AHMAXAAiACwAIAAwAC4AMgA0ACwAIABcACIAUwBoAGUAZQBwAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGUAZQByAFwAIgAsACAAMAAuADIANAAsACAAXAAiAFMAaABlAGUAcABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBhAG0AZQBsAHMAXAAiACwAIAAwAC4AMgA0ACwAIABcACIAUwBoAGUAZQBwAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGwAcABhAGMAYQBzAFwAIgAsACAAMAAuADIANAAsACAAXAAiAFMAaABlAGUAcABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABvAHIAcwBlAHMAXAAiACwAIAAwAC4AMQA5ACwAIABcACIARgBlAGUAZABsAG8AdAAsACAAUABhAHMAdAB1AHIAZQAgAGIAZQBlAGYAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AdQBsAGUAcwAvAGEAcwBzAGUAcwBcACIALAAgADAALgAyADQALAAgAFwAIgBTAGgAZQBlAHAAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAbQB1AHMALwBvAHMAdAByAGkAYwBoAGUAcwBcACIALAAgADAALgAzADYALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAALQAgAG0AZQBhAHQAIABjAGgAaQBjAGsAZQBuAHMAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABuAGkAdAByAG8AZwBlAG4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABmAHIAbwBtACAAdQByAGkAbgBlACAAYQBuAGQAIABmAGEAZQBjAGUAcwAgAGQAZQBwAG8AcwBpAHQAZQBkACAAbwBuACAAcABhAHMAdAB1AHIAZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG4AaQB0AHIAbwBnAGUAbgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGYAcgBvAG0AIAB1AHIAaQBuAGUAIABhAG4AZAAgAGYAYQBlAGMAZQBzACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMARwBBAFMATQBzAG8AaQBsAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4ASAAzAC0ATgAgACsAIABOAE8AeAAtAE4AKQAvAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4ANwAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMgAxACkAOwBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8ATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADQALgA3ADoAIABNAGEAbgB1AHIAZQAgAE0AYQBuAGEAZwBlAG0AZQBuAHQAIAAtACAATwB0AGgAZQByACAATABpAHYAZQBzAHQAbwBjAGsAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADQALgA3AC4AMQAuADEAIABNAGUAdABoAG8AZAAgADEAIAAtACAATQBhAG4AdQByAGUAIABNAGUAdABoAGEAbgBlACAATwB0AGgAZQByACAATABpAHYAZQBzAHQAbwBjAGsAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAFwAbgBUAG8AdABhAGwAIABhAG4AbgB1AGEAbAAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgByAG8AbQAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAG8AZgAgAG8AdABoAGUAcgAgAGwAaQB2AGUAcwB0AG8AYwBrAFwAbgBFAF8AQwBIADQAXABuAHQAIABDAEgANABcAG4ARQBfAHsAQwBIADQAfQA9AFwAXABzAHUAbQBfAGoAXABcAHMAdQBtAF8AbQAoAE4AXwBqAFwAXAB0AGkAbQBlAHMAIABNAF8AagBtAFwAXAB0AGkAbQBlAHMAIAAzADYANQApAFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAbgBOAF8AagAgAD0AIABhAHYAZQByAGEAZwBlACAAYQBuAG4AdQBhAGwAIABuAHUAbQBiAGUAcgAgAG8AZgAgAGwAaQB2AGUAcwB0AG8AYwBrACAAcABlAHIAIABsAGkAdgBlAHMAdABvAGMAawAgAHQAeQBwAGUAIABqACAAKABoAGUAYQBkACkAXABuAE0AXwBqAG0AIAA9ACAAYQBuAG4AdQBhAGwAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABtAGEAbgB1AHIAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIAAoAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGEAbgB1AHIAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABOAF8AagAsACAATQBfAGoAbQAsAFwAbgAgACAAIAAgAFMAVQBNACgATgBfAGoAIAAqACAATQBfAGoAbQAgACoAIAAzADYANQApACAAKgAgADEAMAAgAF4AIAAtADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAG8AdABhAGwAIABhAG4AbgB1AGEAbAAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgByAG8AbQAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAG8AZgAgAG8AdABoAGUAcgAgAGwAaQB2AGUAcwB0AG8AYwBrAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AQwBIADQAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBIADQAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADcALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAxACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AewBDAEgANAB9AD0AXABcAHMAdQBtAFwAXABuAG8AbABpAG0AaQB0AHMAXwBqAFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AbQAoAE4AXwBqAFwAXAB0AGkAbQBlAHMAIABNAF8AagBtAFwAXAB0AGkAbQBlAHMAIAAzADYANQApAFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AXwBqAFwAIgAsACAAXAAiAGEAdgBlAHIAYQBnAGUAIABhAG4AbgB1AGEAbAAgAG4AdQBtAGIAZQByACAAbwBmACAAbABpAHYAZQBzAHQAbwBjAGsAIABwAGUAcgAgAGwAaQB2AGUAcwB0AG8AYwBrACAAdAB5AHAAZQAgAGoAXAAiACwAIABcACIAaABlAGEAZABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AXwBqAG0AXAAiACwAIABcACIAYQBuAG4AdQBhAGwAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABtAGEAbgB1AHIAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAXAAiACwAIABcACIAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAA0AC4ANwAuADEALgAxACwAIAAoADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAagBcACIALAAgAFwAIgBsAGkAdgBlAHMAdABvAGMAawAgAHQAeQBwAGUAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBtAFwAIgAsACAAXAAiAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAHMAeQBzAHQAZQBtAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAxAF8AXwAyAF8AQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABcAG4AQQBuAG4AdQBhAGwAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABtAGEAbgB1AHIAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAXABuAE0AXwBqAG0AXABuAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAbgBNAF8AagBtAD0AVgBTAF8AagBcAFwAdABpAG0AZQBzACAAQgBfAE8AXABcAHQAaQBtAGUAcwAgAE0ATQBTAF8AbQBcAFwAdABpAG0AZQBzACAATQBDAEYAXwBpAG0AXABcAHQAaQBtAGUAcwAgAFwAXAByAGgAbwBcAG4AVgBTAF8AagAgAD0AIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAKABrAGcALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4AQgBfAE8AIAA9ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAcABvAHQAZQBuAHQAaQBhAGwAIAAoAG0AMwAgAEMASAA0AC8AawBnACAAVgBTACkAXABuAE0ATQBTAF8AbQAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIAB3AGEAcwB0AGUAIABpAG4AIABlAGEAYwBoACAAbQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0AXABuAE0AQwBGAF8AaQBtACAAPQAgAG0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIABhAG4AZAAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAHMAeQBzAHQAZQBtAFwAbgByAGgAbwAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAawBnAC8AbQAzACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMQBfAF8AMgBfAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVgBTAF8AagAsACAAQgBfAE8ALAAgAE0ATQBTAF8AbQAsACAATQBDAEYAXwBpAG0ALAAgAHIAaABvACwAXABuACAAIAAgACAAVgBTAF8AagAgACoAIABCAF8ATwAgACoAIABNAE0AUwBfAG0AIAAqACAATQBDAEYAXwBpAG0AIAAqACAAcgBoAG8AXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAxAF8AXwAyAF8AQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBuAG4AdQBhAGwAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABtAGEAbgB1AHIAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADEAXwBfADIAXwBBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGEAbgB1AHIAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAF8AagBtAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAxAF8AXwAyAF8AQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAxAF8AXwAyAF8AQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4ANwAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADIAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMQBfAF8AMgBfAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADEAXwBfADIAXwBBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGEAbgB1AHIAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBfAHsAagBtAH0APQBWAFMAXwBqAFwAXAB0AGkAbQBlAHMAIABCAF8ATwBcAFwAdABpAG0AZQBzACAATQBNAFMAXwBtAFwAXAB0AGkAbQBlAHMAIABNAEMARgBfAHsAaQBtAH0AXABcAHQAaQBtAGUAcwAgAFwAXAByAGgAbwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMQBfAF8AMgBfAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBTAF8AagBcACIALAAgAFwAIgB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAIABwAHIAbwBkAHUAYwB0AGkAbwBuAFwAIgAsACAAXAAiAGsAZwAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAXwBPAFwAIgAsACAAXAAiAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHAAbwB0AGUAbgB0AGkAYQBsAFwAIgAsACAAXAAiAG0AMwAgAEMASAA0AC8AawBnACAAVgBTAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBNAFMAXwBtAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAHcAYQBzAHQAZQAgAGkAbgAgAGUAYQBjAGgAIABtAGEAbgB1AHIAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEMARgBfAGkAbQBcACIALAAgAFwAIgBtAGUAdABoAGEAbgBlACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABzAHQAYQB0AGUAIABhAG4AZAAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAHMAeQBzAHQAZQBtAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAHIAaABvAFwAIgAsACAAXAAiAGQAZQBuAHMAaQB0AHkAIABvAGYAIABtAGUAdABoAGEAbgBlAFwAIgAsACAAXAAiAGsAZwAvAG0AMwBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGkAXAAiACwAIABcACIAcwB0AGEAdABlAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADEAXwBfADIAXwBBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGEAbgB1AHIAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AQQByAGcAdQBtAGUAbgB0AHMAXwBNAGUAdABoAG8AZAAyAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAFMAXwBqAFwAIgAsACAAXAAiAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZAAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AXAAiACwAIABcACIAawBnAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgBfAE8AXAAiACwAIABcACIAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAcABvAHQAZQBuAHQAaQBhAGwAXAAiACwAIABcACIAbQAzACAAQwBIADQALwBrAGcAIABWAFMAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE0AUwBfAG0AXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAdwBhAHMAdABlACAAaQBuACAAZQBhAGMAaAAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAHMAeQBzAHQAZQBtAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQwBGAF8AaQBtAFwAIgAsACAAXAAiAG0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIABhAG4AZAAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAHMAeQBzAHQAZQBtAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAHIAaABvAFwAIgAsACAAXAAiAGQAZQBuAHMAaQB0AHkAIABvAGYAIABtAGUAdABoAGEAbgBlAFwAIgAsACAAXAAiAGsAZwAvAG0AMwBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGkAXAAiACwAIABcACIAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgAsACAAXAAiAGQAZQBnAHIAZQBlAHMAIABDAGUAbABzAGkAdQBzAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBOADIATwBEAGkAcgBlAGMAdAAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ANAAuADcAOgAgAE0AYQBuAHUAcgBlACAATQBhAG4AYQBnAGUAbQBlAG4AdAAgAC0AIABPAHQAaABlAHIAIABMAGkAdgBlAHMAdABvAGMAawBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ANAAuADcALgAxAC4AMwAgAE0AZQB0AGgAbwBkACAAMQAgAC0AIABTAG8AaQBsACAARABpAHIAZQBjAHQAIABOADIATwAgAE8AdABoAGUAcgAgAEwAaQB2AGUAcwB0AG8AYwBrAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMwBfAF8AMQBfAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AUwBvAGkAbABcAG4ARABpAHIAZQBjAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAYQBnAHIAaQBjAHUAbAB0AHUAcgBhAGwAIABzAG8AaQBsAHMAIABmAHIAbwBtACAAZABlAHAAbwBzAGkAdABpAG8AbgAgAG8AZgAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZAB1AG4AZwAgAHQAbwAgAHAAYQBzAHQAdQByAGUAXABuAEUAXwBOADIATwBkAGkAcgBcAG4AdAAgAE4AMgBPAFwAbgBFAF8AewBOADIATwAsAGQAaQByAH0APQBBAEUAXABcAHQAaQBtAGUAcwAgAEUARgBfAHsAUABSAFAAfQBcAFwAdABpAG0AZQBzACAAQwBfAHsATgAyAE8AfQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcAG4AQQBFACAAPQAgAGEAbgBuAHUAYQBsACAAbgBpAHQAcgBvAGcAZQBuACAAZQB4AGMAcgBlAHQAZQBkACAAYgB5ACAAZQBhAGMAaAAgAGwAaQB2AGUAcwB0AG8AYwBrACAAdAB5AHAAZQAgACgAawBnACAATgAvAHkAZQBhAHIAKQBcAG4ARQBGAF8AUABSAFAAIAA9ACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABmAHIAbwBtACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIAB0AG8AIABzAG8AaQBsACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACAAZABlAHAAbwBzAGkAdABlAGQAKQBcAG4AQwBfAE4AMgBPACAAPQAgAGYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMwBfAF8AMQBfAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AUwBvAGkAbABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAEUALAAgAEUARgBfAFAAUgBQACwAIABDAF8ATgAyAE8ALABcAG4AIAAgACAAIABBAEUAIAAqACAARQBGAF8AUABSAFAAIAAqACAAQwBfAE4AMgBPACAAKgAgADEAMAAgAF4AIAAtADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAzAF8AXwAxAF8ARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBTAG8AaQBsAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBEAGkAcgBlAGMAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABhAGcAcgBpAGMAdQBsAHQAdQByAGEAbAAgAHMAbwBpAGwAcwAgAGYAcgBvAG0AIABkAGUAcABvAHMAaQB0AGkAbwBuACAAbwBmACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAdABvACAAcABhAHMAdAB1AHIAZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMwBfAF8AMQBfAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AUwBvAGkAbABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAE4AMgBPAGQAaQByAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAzAF8AXwAxAF8ARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBTAG8AaQBsAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAE4AMgBPAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAzAF8AXwAxAF8ARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBTAG8AaQBsAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgA3AC4AMQAuADMALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAzAF8AXwAxAF8ARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBTAG8AaQBsAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAzAF8AXwAxAF8ARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBTAG8AaQBsAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAHsATgAyAE8ALABkAGkAcgB9AD0AQQBFAFwAXAB0AGkAbQBlAHMAIABFAEYAXwB7AFAAUgBQAH0AXABcAHQAaQBtAGUAcwAgAEMAXwB7AE4AMgBPAH0AXABcAHQAaQBtAGUAcwAgADEAMABeAHsALQAzAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADMAXwBfADEAXwBEAGkAcgBlAGMAdABOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFMAbwBpAGwAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBFAFwAIgAsACAAXAAiAGEAbgBuAHUAYQBsACAAbgBpAHQAcgBvAGcAZQBuACAAZQB4AGMAcgBlAHQAZQBkACAAYgB5ACAAZQBhAGMAaAAgAGwAaQB2AGUAcwB0AG8AYwBrACAAdAB5AHAAZQBcACIALAAgAFwAIgBrAGcAIABOAC8AeQBlAGEAcgBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADQALgA3AC4AMQAuADMALAAgACgAMgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEYAXwBQAFIAUABcACIALAAgAFwAIgBlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGYAcgBvAG0AIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAHQAbwAgAHMAbwBpAGwAXAAiACwAIABcACIAawBnACAATgAyAE8ALQBOAC8AawBnACAATgAgAGQAZQBwAG8AcwBpAHQAZQBkAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBfAE4AMgBPAFwAIgAsACAAXAAiAGYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXAAiACwAIABcACIAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgB6AFwAIgAsACAAXAAiAHcAZQB0ACAAbwByACAAZAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMwBfAF8AMgBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABlAGQAVABvAFAAYQBzAHQAdQByAGUAXABuAEEAbgBuAHUAYQBsACAAbgBpAHQAcgBvAGcAZQBuACAAZQB4AGMAcgBlAHQAZQBkACAAYgB5ACAAbABpAHYAZQBzAHQAbwBjAGsAIAB0AG8AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXABuAEEARQBcAG4AawBnACAATgAvAHkAZQBhAHIAXABuAEEARQA9AFwAXABzAHUAbQBfAGoAKABOAF8AagBcAFwAdABpAG0AZQBzACAATgBFAF8AagBcAFwAdABpAG0AZQBzACAAMwA2ADUAKQBcAG4ATgBfAGoAIAA9ACAAbgB1AG0AYgBlAHIAIABvAGYAIABsAGkAdgBlAHMAdABvAGMAawAgAG8AZgAgAGUAYQBjAGgAIABsAGkAdgBlAHMAdABvAGMAawAgAHQAeQBwAGUAIABqACAAKABoAGUAYQBkACkAXABuAE4ARQBfAGoAIAA9ACAAbgBpAHQAcgBvAGcAZQBuACAAZQB4AGMAcgBlAHQAZQBkACAAYgB5ACAAZQBhAGMAaAAgAGwAaQB2AGUAcwB0AG8AYwBrACAAdAB5AHAAZQAgAGoAIAAoAGsAZwAgAE4ALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAzAF8AXwAyAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGUAZABUAG8AUABhAHMAdAB1AHIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABOAF8AagAsACAATgBFAF8AagAsAFwAbgAgACAAIAAgAE4AXwBqACAAKgAgAE4ARQBfAGoAIAAqACAAMwA2ADUAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAzAF8AXwAyAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGUAZABUAG8AUABhAHMAdAB1AHIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBuAG4AdQBhAGwAIABuAGkAdAByAG8AZwBlAG4AIABlAHgAYwByAGUAdABlAGQAIABiAHkAIABsAGkAdgBlAHMAdABvAGMAawAgAHQAbwAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMwBfAF8AMgBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABlAGQAVABvAFAAYQBzAHQAdQByAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEARQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMwBfAF8AMgBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABlAGQAVABvAFAAYQBzAHQAdQByAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOAC8AeQBlAGEAcgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMwBfAF8AMgBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABlAGQAVABvAFAAYQBzAHQAdQByAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADcALgAxAC4AMwAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAyACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADMAXwBfADIAXwBBAG4AbgB1AGEAbABOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAZQBkAFQAbwBQAGEAcwB0AHUAcgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAzAF8AXwAyAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGUAZABUAG8AUABhAHMAdAB1AHIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEARQA9AFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AagAoAE4AXwBqAFwAXAB0AGkAbQBlAHMAIABOAEUAXwBqAFwAXAB0AGkAbQBlAHMAIAAzADYANQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAzAF8AXwAyAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGUAZABUAG8AUABhAHMAdAB1AHIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAF8AagBcACIALAAgAFwAIgBuAHUAbQBiAGUAcgAgAG8AZgAgAGwAaQB2AGUAcwB0AG8AYwBrACAAbwBmACAAZQBhAGMAaAAgAGwAaQB2AGUAcwB0AG8AYwBrACAAdAB5AHAAZQAgAGoAXAAiACwAIABcACIAaABlAGEAZABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARQBfAGoAXAAiACwAIABcACIAbgBpAHQAcgBvAGcAZQBuACAAZQB4AGMAcgBlAHQAZQBkACAAYgB5ACAAZQBhAGMAaAAgAGwAaQB2AGUAcwB0AG8AYwBrACAAdAB5AHAAZQAgAGoAXAAiACwAIABcACIAawBnACAATgAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGoAXAAiACwAIABcACIAbABpAHYAZQBzAHQAbwBjAGsAIAB0AHkAcABlAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ANAAuADcAOgAgAE0AYQBuAHUAcgBlACAATQBhAG4AYQBnAGUAbQBlAG4AdAAgAC0AIABPAHQAaABlAHIAIABMAGkAdgBlAHMAdABvAGMAawBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ANAAuADcALgAxAC4ANQAgAE0AZQB0AGgAbwBkACAAMQAgAC0AIABTAG8AaQBsACAAQQB0AG0AbwBzAHAAaABlAHIAaQBjACAARABlAHAAbwBzAGkAdABpAG8AbgAgAE4AMgBPACAATwB0AGgAZQByACAATABpAHYAZQBzAHQAbwBjAGsAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA1AF8AXwAxAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAFwAbgBBAHQAbQBvAHMAcABoAGUAcgBpAGMAIABkAGUAcABvAHMAaQB0AGkAbwBuACAAZQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlAFwAbgBFAF8ATgAyAE8AYQBkAFwAbgB0ACAATgAyAE8AXABuAEUAXwB7AE4AMgBPACwAYQBkAH0APQBNAF8AewB2AG8AbAB9AFwAXAB0AGkAbQBlAHMAIABFAEYAXwB7AE4AMgBPAH0AXABcAHQAaQBtAGUAcwAgAEMAXwB7AE4AMgBPAH0AXABcAHQAaQBtAGUAcwAgADEAMABeAHsALQAzAH0AXABuAE0AXwB2AG8AbAAgAD0AIABtAGEAcwBzACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAZgByAG8AbQAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZgBhAGUAYwBlAHMAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUAIAAoAGsAZwAgAE4AKQBcAG4ARQBGAF8ATgAyAE8AIAA9ACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGEAdABtAG8AcwBwAGgAZQByAGkAYwAgAGQAZQBwAG8AcwBpAHQAaQBvAG4AIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQBcAG4AQwBfAE4AMgBPACAAPQAgAGYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANQBfAF8AMQBfAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AUABhAHMAdAB1AHIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAF8AdgBvAGwALAAgAEUARgBfAE4AMgBPACwAIABDAF8ATgAyAE8ALABcAG4AIAAgACAAIABNAF8AdgBvAGwAIAAqACAARQBGAF8ATgAyAE8AIAAqACAAQwBfAE4AMgBPACAAKgAgADEAMAAgAF4AIAAtADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA1AF8AXwAxAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHQAbQBvAHMAcABoAGUAcgBpAGMAIABkAGUAcABvAHMAaQB0AGkAbwBuACAAZQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA1AF8AXwAxAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8ATgAyAE8AYQBkAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA1AF8AXwAxAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAE4AMgBPAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA1AF8AXwAxAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgA3AC4AMQAuADUALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA1AF8AXwAxAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA1AF8AXwAxAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAHsATgAyAE8ALABhAGQAfQA9AE0AXwB7AHYAbwBsAH0AXABcAHQAaQBtAGUAcwAgAEUARgBfAHsATgAyAE8AfQBcAFwAdABpAG0AZQBzACAAQwBfAHsATgAyAE8AfQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANQBfAF8AMQBfAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AUABhAHMAdAB1AHIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAF8AdgBvAGwAXAAiACwAIABcACIAbQBhAHMAcwAgAG8AZgAgAG4AaQB0AHIAbwBnAGUAbgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGYAcgBvAG0AIAB1AHIAaQBuAGUAIABhAG4AZAAgAGYAYQBlAGMAZQBzACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAGsAZwAgAE4AXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAA0AC4ANwAuADEALgA1ACwAIAAoADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAF8ATgAyAE8AXAAiACwAIABcACIAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGEAdABtAG8AcwBwAGgAZQByAGkAYwAgAGQAZQBwAG8AcwBpAHQAaQBvAG4AXAAiACwAIABcACIAawBnACAATgAyAE8ALQBOAC8AawBnACAATgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAXwBOADIATwBcACIALAAgAFwAIgBmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAagBcACIALAAgAFwAIgBwAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBpAFwAIgAsACAAXAAiAGkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAHIAXAAiACwAIABcACIAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBWAG8AbABhAHQAaQBsAGkAcwBlAGQARgByAG8AbQBQAGEAcwB0AHUAcgBlAFwAbgBNAGEAcwBzACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAZgByAG8AbQAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZgBhAGUAYwBlAHMAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUAXABuAE0AXwB2AG8AbABcAG4AawBnACAATgBcAG4ATQBfAHsAdgBvAGwAfQA9AEEARQBcAFwAdABpAG0AZQBzACAARgByAGEAYwBHAEEAUwBNAHMAbwBpAGwAXABuAEEARQAgAD0AIABhAG4AbgB1AGEAbAAgAG4AaQB0AHIAbwBnAGUAbgAgAGUAeABjAHIAZQB0AGUAZAAgAGIAeQAgAGUAYQBjAGgAIABsAGkAdgBlAHMAdABvAGMAawAgAHQAeQBwAGUAIAAoAGsAZwAgAE4ALwB5AGUAYQByACkAXABuAEYAcgBhAGMARwBBAFMATQBzAG8AaQBsACAAPQAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG4AaQB0AHIAbwBnAGUAbgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGYAcgBvAG0AIAB1AHIAaQBuAGUAIABhAG4AZAAgAGYAYQBlAGMAZQBzACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlACAAKAAoAGsAZwAgAE4ASAAzAC0ATgAgACsAIABOAE8AeAAtAE4AKQAvAGsAZwAgAE4AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA1AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAFYAbwBsAGEAdABpAGwAaQBzAGUAZABGAHIAbwBtAFAAYQBzAHQAdQByAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQBFACwAIABGAHIAYQBjAEcAQQBTAE0AcwBvAGkAbAAsAFwAbgAgACAAIAAgAEEARQAgACoAIABGAHIAYQBjAEcAQQBTAE0AcwBvAGkAbABcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADUAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0AUABhAHMAdAB1AHIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAHMAcwAgAG8AZgAgAG4AaQB0AHIAbwBnAGUAbgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGYAcgBvAG0AIAB1AHIAaQBuAGUAIABhAG4AZAAgAGYAYQBlAGMAZQBzACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA1AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAFYAbwBsAGEAdABpAGwAaQBzAGUAZABGAHIAbwBtAFAAYQBzAHQAdQByAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AXwB2AG8AbABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBWAG8AbABhAHQAaQBsAGkAcwBlAGQARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBWAG8AbABhAHQAaQBsAGkAcwBlAGQARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgA3AC4AMQAuADUALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMgApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA1AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAFYAbwBsAGEAdABpAGwAaQBzAGUAZABGAHIAbwBtAFAAYQBzAHQAdQByAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADUAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0AUABhAHMAdAB1AHIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AXwB7AHYAbwBsAH0APQBBAEUAXABcAHQAaQBtAGUAcwAgAEYAcgBhAGMARwBBAFMATQBzAG8AaQBsAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA1AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAFYAbwBsAGEAdABpAGwAaQBzAGUAZABGAHIAbwBtAFAAYQBzAHQAdQByAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBFAFwAIgAsACAAXAAiAGEAbgBuAHUAYQBsACAAbgBpAHQAcgBvAGcAZQBuACAAZQB4AGMAcgBlAHQAZQBkACAAYgB5ACAAZQBhAGMAaAAgAGwAaQB2AGUAcwB0AG8AYwBrACAAdAB5AHAAZQBcACIALAAgAFwAIgBrAGcAIABOAC8AeQBlAGEAcgBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAYgB5ACAANAAuADcALgAxAC4AMwAsACAAKAAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAcgBhAGMARwBBAFMATQBzAG8AaQBsAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG4AaQB0AHIAbwBnAGUAbgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGYAcgBvAG0AIAB1AHIAaQBuAGUAIABhAG4AZAAgAGYAYQBlAGMAZQBzACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiACgAawBnACAATgBIADMALQBOACAAKwAgAE4ATwB4AC0ATgApAC8AawBnACAATgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8ATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA0AC4ANwA6ACAATQBhAG4AdQByAGUAIABNAGEAbgBhAGcAZQBtAGUAbgB0ACAALQAgAE8AdABoAGUAcgAgAEwAaQB2AGUAcwB0AG8AYwBrAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA0AC4ANwAuADEALgA3ACAATQBlAHQAaABvAGQAIAAxACAALQAgAFMAbwBpAGwAIABMAGUAYQBjAGgAaQBuAGcAIABBAG4AZAAgAFIAdQBuAG8AZgBmACAATgAyAE8AIABPAHQAaABlAHIAIABMAGkAdgBlAHMAdABvAGMAawBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADcAXwBfADEAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAFwAbgBMAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmACAAZQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlAFwAbgBFAF8ATgAyAE8AbABlAGEAYwBoAFwAbgB0ACAATgAyAE8AXABuAEUAXwB7AE4AMgBPACwAbABlAGEAYwBoAH0APQBNAF8AewBsAGUAYQBjAGgAfQBcAFwAdABpAG0AZQBzACAARQBGAF8AewBsAGUAYQBjAGgAfQBcAFwAdABpAG0AZQBzACAAQwBfAHsATgAyAE8AfQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcAG4ATQBfAGwAZQBhAGMAaAAgAD0AIABtAGEAcwBzACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAbABvAHMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoAGsAZwAgAE4AKQBcAG4ARQBGAF8AbABlAGEAYwBoACAAPQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACkAXABuAEMAXwBOADIATwAgAD0AIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADcAXwBfADEAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AXwBsAGUAYQBjAGgALAAgAEUARgBfAGwAZQBhAGMAaAAsACAAQwBfAE4AMgBPACwAXABuACAAIAAgACAATQBfAGwAZQBhAGMAaAAgACoAIABFAEYAXwBsAGUAYQBjAGgAIAAqACAAQwBfAE4AMgBPACAAKgAgADEAMAAgAF4AIAAtADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA3AF8AXwAxAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AUABhAHMAdAB1AHIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgAgAGUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZAB1AG4AZwAgAGQAZQBwAG8AcwBpAHQAZQBkACAAbwBuACAAcABhAHMAdAB1AHIAZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANwBfAF8AMQBfAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFAAYQBzAHQAdQByAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwBOADIATwBsAGUAYQBjAGgAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADcAXwBfADEAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAE4AMgBPAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA3AF8AXwAxAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AUABhAHMAdAB1AHIAZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4ANwAuADEALgA3ACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADEAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANwBfAF8AMQBfAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFAAYQBzAHQAdQByAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADcAXwBfADEAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAHsATgAyAE8ALABsAGUAYQBjAGgAfQA9AE0AXwB7AGwAZQBhAGMAaAB9AFwAXAB0AGkAbQBlAHMAIABFAEYAXwB7AGwAZQBhAGMAaAB9AFwAXAB0AGkAbQBlAHMAIABDAF8AewBOADIATwB9AFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA3AF8AXwAxAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AUABhAHMAdAB1AHIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAF8AbABlAGEAYwBoAFwAIgAsACAAXAAiAG0AYQBzAHMAIABvAGYAIABuAGkAdAByAG8AZwBlAG4AIABsAG8AcwB0ACAAdABvACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIALAAgAFwAIgBrAGcAIABOAFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAANAAuADcALgAxAC4ANwAsACAAKAAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBfAGwAZQBhAGMAaABcACIALAAgAFwAIgBlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIALAAgAFwAIgBrAGcAIABOADIATwAtAE4ALwBrAGcAIABOAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBfAE4AMgBPAFwAIgAsACAAXAAiAGYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXAAiACwAIABcACIAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAFwAbgBNAGEAcwBzACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAbABvAHMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAE0AXwBsAGUAYQBjAGgAXABuAGsAZwAgAE4AXABuAE0AXwB7AGwAZQBhAGMAaAB9AD0AQQBFAFwAXAB0AGkAbQBlAHMAIABGAHIAYQBjAFcAZQB0AFwAXAB0AGkAbQBlAHMAIABGAHIAYQBjAEwARQBBAEMASABcAG4AQQBFACAAPQAgAGEAbgBuAHUAYQBsACAAbgBpAHQAcgBvAGcAZQBuACAAZQB4AGMAcgBlAHQAZQBkACAAYgB5ACAAZQBhAGMAaAAgAGwAaQB2AGUAcwB0AG8AYwBrACAAdAB5AHAAZQAgACgAawBnACAATgAvAHkAZQBhAHIAKQBcAG4ARgByAGEAYwBXAGUAdAAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABuAGkAdAByAG8AZwBlAG4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ARgByAGEAYwBMAEUAQQBDAEgAIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAYQBsAGwAIABuAGkAdAByAG8AZwBlAG4AIAB0AGgAYQB0ACAAaQBzACAAbABvAHMAdAAgAHQAaAByAG8AdQBnAGgAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEEARQAsACAARgByAGEAYwBXAGUAdAAsACAARgByAGEAYwBMAEUAQQBDAEgALABcAG4AIAAgACAAIABBAEUAIAAqACAARgByAGEAYwBXAGUAdAAgACoAIABGAHIAYQBjAEwARQBBAEMASABcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAcwBzACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAbABvAHMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAF8AbABlAGEAYwBoAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA3AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABvAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgA3AC4AMQAuADcALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMgApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA3AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABvAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANwBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAbwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAF8AewBsAGUAYQBjAGgAfQA9AEEARQBcAFwAdABpAG0AZQBzACAARgByAGEAYwBXAGUAdABcAFwAdABpAG0AZQBzACAARgByAGEAYwBMAEUAQQBDAEgAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEARQBcACIALAAgAFwAIgBhAG4AbgB1AGEAbAAgAG4AaQB0AHIAbwBnAGUAbgAgAGUAeABjAHIAZQB0AGUAZAAgAGIAeQAgAGUAYQBjAGgAIABsAGkAdgBlAHMAdABvAGMAawAgAHQAeQBwAGUAXAAiACwAIABcACIAawBnACAATgAvAHkAZQBhAHIAXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGIAeQAgADQALgA3AC4AMQAuADMALAAgACgAMgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAHIAYQBjAFcAZQB0AFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG4AaQB0AHIAbwBnAGUAbgAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAYQBsAGwAIABuAGkAdAByAG8AZwBlAG4AIAB0AGgAYQB0ACAAaQBzACAAbABvAHMAdAAgAHQAaAByAG8AdQBnAGgAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAegBcACIALAAgAFwAIgBsAG8AYwBhAHQAaQBvAG4AIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAagBcACIALAAgAFwAIgBwAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBpAHIAXAAiACwAIABcACIAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AIgB9AF0ALAAiAHAAcgBvAGoAZQBjAHQATgBhAG0AZQBzACIAOgBbACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFYAYQBpAHIAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE8AbgBlAEMAbwBsAHUAbQBuAEEAbgBkAEgAZQBhAGQAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAATgAyAE8ARQBGAEYAcgBvAG0AUAByAG8AZABJAHIAcgBpAGcAYQB0AGkAbwBuAFIAYQBpAG4AZgBhAGwAbAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AQwBvAG4AdgBlAHIAdABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBUAG8AQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADEAXwAyACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAzAF8ANAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVAAiACwAIgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBIAGEAcgB2AGUAcwB0AEkAbgBkAGUAeAAiACwAIgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvACIALAAiAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEMAYQBsAGMAdQBsAGEAdABlAEYAcgBhAGMAdABpAG8AbgBSAGUAcwBpAGQAdQBlAFIAZQBtAG8AdgBlAGQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAUAByAG8AZAB1AGMAZQBkAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFAAcgBvAGQAdQBjAGUAZABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBQAHIAbwBkAHUAYwBlAGQAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFAAcgBvAGQAdQBjAGUAZABfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFAAcgBvAGQAdQBjAGUAZABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFAAcgBvAGQAdQBjAGUAZABfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAZQBkAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGUAZABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABlAGQAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGUAZABfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGUAZABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGUAZABfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBBAHYAZQByAGEAZwBlAEwAaQB2AGUAdwBlAGkAZwBoAHQAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBBAHYAZQByAGEAZwBlAEwAaQB2AGUAdwBlAGkAZwBoAHQAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBBAHYAZQByAGEAZwBlAEwAaQB2AGUAdwBlAGkAZwBoAHQAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AQQB2AGUAcgBhAGcAZQBMAGkAdgBlAHcAZQBpAGcAaAB0AF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBBAHYAZQByAGEAZwBlAEwAaQB2AGUAdwBlAGkAZwBoAHQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAEEAdgBlAHIAYQBnAGUATABpAHYAZQB3AGUAaQBnAGgAdABfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBGAHIAYQBjAHQAaQBvAG4AVwBhAHMAdABlAEkAbgBNAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAEYAcgBhAGMAdABpAG8AbgBXAGEAcwB0AGUASQBuAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ARgByAGEAYwB0AGkAbwBuAFcAYQBzAHQAZQBJAG4ATQBNAFMAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ARgByAGEAYwB0AGkAbwBuAFcAYQBzAHQAZQBJAG4ATQBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAEYAcgBhAGMAdABpAG8AbgBXAGEAcwB0AGUASQBuAE0ATQBTAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBGAHIAYQBjAHQAaQBvAG4AVwBhAHMAdABlAEkAbgBNAE0AUwBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAEMAbwBuAHYAZQByAHMAaQBvAG4ARgBhAGMAdABvAHIAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAEMAbwBuAHYAZQByAHMAaQBvAG4ARgBhAGMAdABvAHIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAEMAbwBuAHYAZQByAHMAaQBvAG4ARgBhAGMAdABvAHIAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATQBlAHQAaABhAG4AZQBDAG8AbgB2AGUAcgBzAGkAbwBuAEYAYQBjAHQAbwByAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAEMAbwBuAHYAZQByAHMAaQBvAG4ARgBhAGMAdABvAHIAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAE0AZQB0AGgAYQBuAGUAQwBvAG4AdgBlAHIAcwBpAG8AbgBGAGEAYwB0AG8AcgBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAEQAYQB0AGEAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGEAbgB1AHIAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGEAbgB1AHIAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMQBfAF8AMgBfAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAxAF8AXwAyAF8AQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADEAXwBfADIAXwBBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGEAbgB1AHIAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMQBfAF8AMgBfAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBVAG4AaQB0ACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMQBfAF8AMgBfAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADEAXwBfADIAXwBBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGEAbgB1AHIAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAxAF8AXwAyAF8AQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAxAF8AXwAyAF8AQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMQBfAF8AMgBfAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwBfAE0AZQB0AGgAbwBkADIAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8ATgAyAE8ARABpAHIAZQBjAHQALgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAzAF8AXwAxAF8ARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBTAG8AaQBsACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAGkAbABfAE4AMgBPAEQAaQByAGUAYwB0AC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMwBfAF8AMQBfAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AUwBvAGkAbABfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBOADIATwBEAGkAcgBlAGMAdAAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADMAXwBfADEAXwBEAGkAcgBlAGMAdABOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFMAbwBpAGwAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8ATgAyAE8ARABpAHIAZQBjAHQALgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAzAF8AXwAxAF8ARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBTAG8AaQBsAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBOADIATwBEAGkAcgBlAGMAdAAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADMAXwBfADEAXwBEAGkAcgBlAGMAdABOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFMAbwBpAGwAXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBOADIATwBEAGkAcgBlAGMAdAAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADMAXwBfADEAXwBEAGkAcgBlAGMAdABOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFMAbwBpAGwAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBOADIATwBEAGkAcgBlAGMAdAAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADMAXwBfADEAXwBEAGkAcgBlAGMAdABOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFMAbwBpAGwAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAGkAbABfAE4AMgBPAEQAaQByAGUAYwB0AC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMwBfAF8AMQBfAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AUwBvAGkAbABfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAGkAbABfAE4AMgBPAEQAaQByAGUAYwB0AC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMwBfAF8AMgBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABlAGQAVABvAFAAYQBzAHQAdQByAGUAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8ATgAyAE8ARABpAHIAZQBjAHQALgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAzAF8AXwAyAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGUAZABUAG8AUABhAHMAdAB1AHIAZQBfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBOADIATwBEAGkAcgBlAGMAdAAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADMAXwBfADIAXwBBAG4AbgB1AGEAbABOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAZQBkAFQAbwBQAGEAcwB0AHUAcgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAGkAbABfAE4AMgBPAEQAaQByAGUAYwB0AC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMwBfAF8AMgBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABlAGQAVABvAFAAYQBzAHQAdQByAGUAXwBVAG4AaQB0ACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAGkAbABfAE4AMgBPAEQAaQByAGUAYwB0AC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMwBfAF8AMgBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABlAGQAVABvAFAAYQBzAHQAdQByAGUAXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBOADIATwBEAGkAcgBlAGMAdAAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADMAXwBfADIAXwBBAG4AbgB1AGEAbABOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAZQBkAFQAbwBQAGEAcwB0AHUAcgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8ATgAyAE8ARABpAHIAZQBjAHQALgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAzAF8AXwAyAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGUAZABUAG8AUABhAHMAdAB1AHIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8ATgAyAE8ARABpAHIAZQBjAHQALgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAzAF8AXwAyAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGUAZABUAG8AUABhAHMAdAB1AHIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAGkAbABfAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANQBfAF8AMQBfAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AUABhAHMAdAB1AHIAZQAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADUAXwBfADEAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFAAYQBzAHQAdQByAGUAXwBUAGkAdABsAGUAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ALgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA1AF8AXwAxAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAGkAbABfAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANQBfAF8AMQBfAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AUABhAHMAdAB1AHIAZQBfAFUAbgBpAHQAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ALgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA1AF8AXwAxAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8AUwBvAHUAcgBjAGUAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ALgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA1AF8AXwAxAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ALgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA1AF8AXwAxAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADUAXwBfADEAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFAAYQBzAHQAdQByAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADUAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0AUABhAHMAdAB1AHIAZQAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADUAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0AUABhAHMAdAB1AHIAZQBfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADUAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0AUABhAHMAdAB1AHIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADUAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0AUABhAHMAdAB1AHIAZQBfAFUAbgBpAHQAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ALgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA1AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAFYAbwBsAGEAdABpAGwAaQBzAGUAZABGAHIAbwBtAFAAYQBzAHQAdQByAGUAXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADUAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0AUABhAHMAdAB1AHIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAGkAbABfAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBWAG8AbABhAHQAaQBsAGkAcwBlAGQARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADUAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0AUABhAHMAdAB1AHIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAGkAbABfAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADcAXwBfADEAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAGkAbABfAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADcAXwBfADEAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAGkAbABfAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADcAXwBfADEAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAGkAbABfAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADcAXwBfADEAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYALgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA3AF8AXwAxAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AUABhAHMAdAB1AHIAZQBfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAGkAbABfAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADcAXwBfADEAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANwBfAF8AMQBfAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFAAYQBzAHQAdQByAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAGkAbABfAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADcAXwBfADEAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANwBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAbwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANwBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAbwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBUAGkAdABsAGUAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANwBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAbwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANwBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAbwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBVAG4AaQB0ACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAGkAbABfAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AUwBvAHUAcgBjAGUAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANwBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAbwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYALgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA3AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABvAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANwBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAbwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBBAHIAZwB1AG0AZQBuAHQAcwAiAF0ALAAiAGwAbwBjAGEAbABlACIAOgB7ACIAbABpAHMAdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHIAbwB3AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiADsAIgAsACIAYwBvAGwAdQBtAG4AUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgB0AGgAbwB1AHMAYQBuAGQAcwBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFAAbwBzAGkAdABpAG8AbgBzACIAOgBbADMAXQAsACIAZABlAGMAaQBtAGEAbABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAuACIALAAiAGQAYQB0AGUATwByAGQAZQByACIAOgAiAEQATQBZACIALAAiAGMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbAAiADoAIgAkACIALAAiAGkAcwBDAHUAcgByAGUAbgBjAHkAUwB5AG0AYgBvAGwATABlAGEAZAAiADoAdAByAHUAZQAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAGUAcABCAHkAUwBwAGEAYwBlACIAOgBmAGEAbABzAGUALAAiAHIAbwB3AEwAZQB0AHQAZQByACIAOgAiAFIAIgAsACIAYwBvAGwAdQBtAG4ATABlAHQAdABlAHIAIgA6ACIAQwAiACwAIgByAGMATABlAGYAdABCAHIAYQBjAGsAZQB0ACIAOgAiAFsAIgAsACIAcgBjAFIAaQBnAGgAdABCAHIAYQBjAGsAZQB0ACIAOgAiAF0AIgAsACIAcwB0AGEAdABlAG0AZQBuAHQAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBsAG8AYwBhAGwAZQBOAGEAbQBlACIAOgAiAGUAbgAtAHUAcwAiAH0AfQA=</AFEJSONBlob>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ACB660BB23738846A00119B5826AC974" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3e3613359d4ae7f6bda6c57be713f101">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7291119c-fce9-4911-96ae-b800be5dccd8" xmlns:ns3="09eef6d6-daa8-4301-8f9f-b1ec38079286" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87491bfad7f11426ad96486e70428b3e" ns2:_="" ns3:_="">
     <xsd:import namespace="7291119c-fce9-4911-96ae-b800be5dccd8"/>
@@ -30005,20 +30009,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgAFwAdQAwADAAMgA3AEYAcgB5AFwAdQAwADAAMgA3ACAAdABvACAAXAB1ADAAMAAyADcARAByAHkAXAB1ADAAMAAyADcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADIAMAAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0AGUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFQAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAUAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEUAVAAgAD0AIABwAG8AdABlAG4AdABpAGEAbAAgAGUAdgBhAHAAbwB0AHIAYQBuAHMAcABpAHIAYQB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAE0AQQBUACAAbQBpAG4AIABhAG4AZAAgAE0AQQBUACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AZQBkAGkAYQBuACAAQQBuAG4AdQBhAGwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAAoAE0AQQBUACkAXAAiACwAIABcACIATQBpAG4AIABNAEEAVABcACIALAAgAFwAIgBNAGEAeAAgAE0AQQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiIAAyADYAIABDAFwAIgAsACAAMgA2ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgAFwAIgAxADUAIAAtACAAMgA1ACAAQwBcACIALAAgADEANQAsACAAMgA1AC4AOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIiAAMQA0ACAAQwBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEANAAuADkAOQA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABaAG8AbgBlAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAXAB1ADAAMAAzAGUAIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAXAB1ADAAMAAzAGUAowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoADMALgBEAC4AYgAuADIAKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAMAAuADIANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AIAAzAC4ARAAuAEIAXwAxADAAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAGwAZQBhAGMAaABcACIALAAwAC4AMAAxADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcAG4ATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADUALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAGoAXAAiACwAXAAiAEUARgBOADIATwBcACIALAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5AFwAIgAsACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAA1ADkALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAXAAiACwAMAAuADAAMAA3ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABsAG8AdwAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAMgA5ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAOAAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAMAAuADAAMQA5ADkALAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsADAALgAwADAANQAzACwAIABcACIAQwBvAHQAdABvAG4AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAMAAuADAAMAA2ADQALAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABjAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnACkAXAAiACwAMAAuADAAMAAzACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBDAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABzAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnACkAXAAiACwAMAAuADAAMAA1ACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBTAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAMAAuADAAMAAyADYALAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABkAHUAcABsAGkAYwBhAHQAZQAgAFwAdQAwADAAMgA3AEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcAHUAMAAwADIANwAsACAAXAB1ADAAMAAyADcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcAHUAMAAwADIANwAgAGEAbgBkACAAXAB1ADAAMAAyADcAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AG4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAdQAwADAAMgA3ACAAcgBvAHcAIAB3AGkAdABoACAAcwBhAG0AZQAgAEUARgAgAGYAbwByACAAbABvAHcAIABhAG4AZAAgAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXABuAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXABuAEkAUABDAEMAOgAgAE4AMgBPACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATQBBAE4AQQBHAEUARAAgAFMATwBJAEwAUwAsACAAQQBOAEQAIABDAE8AMgAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAEwASQBNAEUAIABBAE4ARAAgAFUAUgBFAEEAIABBAFAAUABMAEkAQwBBAFQASQBPAE4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAFcARQBUACAAZgBvAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEkAUABDAEMAIAAyADAAMQA5ACAAUgBlAGYAaQBuAGUAbQBlAG4AdAAgAFYAbwBsAHUAbQBlACAANAA6ACAAQwBoAGEAcAB0AGUAcgAgADEAMQA6ACAATgAyAE8AIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAGEAbgBhAGcAZQBkACAAUwBvAGkAbABzACwAIABhAG4AZAAgAEMATwAyACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATABpAG0AZQAgAGEAbgBkACAAVQByAGUAYQAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlACAAaQByAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBwAHIAaQBuAGsAbABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAcgBmAGEAYwBlACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABUAGEAYgBsAGUAIABjAHIAZQBhAHQAZQBkACAAYgBhAHMAZQBkACAAbwBuACAAVgBFAEUAUgBHACAAdABlAHgAdAAgAFwAdQAwADAAMgA3AEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuAFwAdQAwADAAMgA3AFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAOgAgAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAFAAUgBQACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAFAAUgBQAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAB1ADAAMAAyADcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAdQAwADAAMgA3ACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AbwBuAHQAaABzACAAdABvACAAUwBlAGEAcwBvAG4AcwAgAE0AYQBwAHAAaQBuAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AbgB0AGgAXAAiACwAIABcACIAUwBlAGEAcwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAYQBuAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBiAHIAdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHIAYwBoAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHAAcgBpAGwAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQB5AFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbgBlAFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbAB5AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAZwB1AHMAdABcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAHAAdABlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AYwB0AG8AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB2AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGMAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAbgB1AHIAZQAgAE0AYQBuAGEAZwBlAG0AZQBuAHQAIAATICAATQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHAAZQByACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGkAbQApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA4AC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAyACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAIAAoALoAQwApAFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAUwBsAHUAcgByAHkAIAAoAHcAaQB0AGgAbwB1AHQAIABuAGEAdAB1AHIAYQBsACAAYwByAHUAcwB0ACkAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAGIAKQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABTAHQAbwByAGEAZwBlACAAXAB1ADAAMAAzAGMAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AFAAbwB1AGwAdAByAHkAIAB3AGkAdABoACAAYQBuAGQAIAB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABzAGUAcABhAHIAYQB0AGUAIABOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE0AQQBUACAAcgBhAHcAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAbABsAG8AdwAgAGwAbwBvAGsAdQBwACAAbwBmACAAbgB1AG0AYgBlAHIAcwAuAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBuAGQAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAcgBlAHQAdQByAG4AZQBkACAAdABvACAAdABoAGUAIABzAG8AaQBsAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AaQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADEALgA0AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBOAGkAIABcAHUAMAAwADIANgAgAEUARgBOADIATwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAE4AMgBPACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUATgAyAE8AOgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXABuAEcAVwBQAE4AMgBPADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBOADIATwAsACAARwBXAFAAXwBOADIATwAsAFwAbgAgACAAIAAgAEUAXwBOADIATwAgACoAIABHAFcAUABfAE4AMgBPAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAE4AMgBPACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AE4AMgBPAH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AE4AMgBPAH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBOADIATwBcACIALABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAATgAyAE8AXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAEMASAA0ACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUAQwBIADQAOgAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXABuAEcAVwBQAEMASAA0ADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBDAEgANAAsACAARwBXAFAAXwBDAEgANAAsAFwAbgAgACAAIAAgAEUAXwBDAEgANAAgACoAIABHAFcAUABfAEMASAA0AFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEMASAA0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AEMASAA0AH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AEMASAA0AH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBDAEgANABcACIALABcACIATQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAAQwBIADQAXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAbABpAHYAZQBzAHQAbwBjAGsAIAB0AHkAcABlAHMAXABuAEUAeABjAGUAbAAgAG0AbwBkAHUAbABlACAAbgBhAG0AZQA6ACAAUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBcAG4ARgByAGEAYwBXAEUAVABNAE0AUwBpACAAPQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4AKABUAGEAYgBsAGUAIABBADUALgA1AC4AMQAwAC4AMgAgAGkAcwAgAHIAZQBmAGUAcgBlAG4AYwBlAGQAIABpAG4AIABOAEkAUgAgAGIAdQB0ACAAMQAgAGkAcwAgAHUAcwBlAGQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAxACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXABuAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTACAAPQAgADAALgAwADIAIAAoAEcAZwAgAE4ALwBHAGcAIABhAHAAcABsAGkAZQBkACkAIAAoAEMAUwAgAEUARgAsACAAcwBvAHUAcgBjAGUAIABJAFAAQwBDACAAKAAyADAAMQA5ACkAKQAgAFwAbgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAbABvAHMAdAAgAHQAaAByAG8AdQBnAGgAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAIAAwAC4AMAAwADUAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsACAAMAAuADAAMAA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAgADAALgAwADAAMQA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcABcACIALAAgADAALgAwADAANAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAIABjAGEAbgBlAFwAIgAsACAAMAAuADAAMQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAMAAuADAAMAA1ADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAMAAuADAAMAA2ADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXABuAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVgBhAGkAcgBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE0AUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAAVABhAGIAbABlACAANQAuADEAMgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAOQAsACAAMwAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AG0AYgBvAGwAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgAgACgAbQA9ADEAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADIAXAAiACwAIABcACIATABpAHEAdQBpAGQAIABzAHkAcwB0AGUAbQBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwAgACgAbQA9ADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAG0APQAzACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGEAXAAiACwAIABcACIAUwB1AG0AcAAgAGEAbgBkACAAZABpAHMAcABlAHIAcwBhAGwAIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtACAAKABtAD0AMwBhACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGIAXAAiACwAIABcACIARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAEQAcgBhAGkAbgBzACAAdABvACAAcABhAGQAZABvAGMAawAgACgAbQA9ADMAYgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIANABcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAIAAoAG0APQA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA1AFwAIgAsACAAXAAiAEQAcgB5AGwAbwB0ACAAKABmAGUAZQBkACAAcABhAGQAKQBcACIALAAgAFwAIgBEAHIAeQBsAG8AdAAgACgAZgBlAGUAZAAgAHAAYQBkACkAIAAoAG0APQA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA2AFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQAgACgAbQA9ADYAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADcAXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwAgACgAbQA9ADcAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADgAXAAiACwAIABcACIARABlAGUAcAAgAGwAaQB0AHQAZQByAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgAgACgAbQA9ADgAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADkAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQAgACgAbQA9ADkAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMABcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwAgACgAbQA9ADEAMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnACAAKABtAD0AMQAxACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADEAYQBcACIALAAgAFwAIgBCAGUAbAB0ACAAbQBhAG4AdQByAGUAIAByAGUAbQBvAHYAYQBsAFwAIgAsACAAXAAiAEIAZQBsAHQAIABtAGEAbgB1AHIAZQAgAHIAZQBtAG8AdgBhAGwAIAAoAG0APQAxADEAYQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAGIAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABzAHQAbwByAGUAZAAgAGkAbgAgAGgAbwB1AHMAZQBcACIALAAgAFwAIgBNAGEAbgB1AHIAZQAgAHMAdABvAHIAZQBkACAAaQBuACAAaABvAHUAcwBlACAAKABtAD0AMQAxAGIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAKABtAD0AMQAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADMAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAG0APQAxADMAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEANABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAIAAoAG0APQAxADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQgBlAGUAZgAgAGMAYQB0AHQAbABlACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAYQB0AHQAbABlACwAIABmAG8AcgAgAG0AYQBuAHUAZgBhAGMAdAB1AHIAaQBuAGcAIABiAGUAZQBmAFwAIgAsACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBhAHQAdABsAGUALAAgAGYAbwByACAAcAByAGkAbQBlACAAYgBlAGUAZgBcACIALAAgAFwAIgBOAFMAVwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAYQB0AHQAbABlACwAIAB3AGUAYQBuAGUAcgBzAFwAIgAsACAAXAAiAE4AVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFEATABEAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAVABBAFMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBWAEkAQwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFcAQQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBDAGgAaQBjAGsAZQBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEMAaABpAGMAawBlAG4AcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBoAGkAYwBrAGUAbgBzACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQwBoAGkAYwBrAGUAbgBzAF8AVgBhAGkAcgBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEMAaABpAGMAawBlAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQwBoAGkAYwBrAGUAbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBDAGgAaQBjAGsAZQBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAG8AZAB1AGMAdABcACIALAAgAFwAIgBTAG8AdQByAGMAZQAgAHIAZQBnAGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBoAGkAYwBrAGUAbgBzAFwAIgAsACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEQAYQBpAHIAeQBjAGEAdAB0AGwAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABwAHIAbwBkAHUAYwB0AHMAIABmAG8AcgAgAHMAYwBvAHAAZQAgADMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXwBWAGEAaQByAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8ARABhAGkAcgB5AGMAYQB0AHQAbABlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATABpAGYAZQBjAHkAYwBsAGUAcwAuACAAKAAyADAAMgA2ACkALgAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABHAGEAcwAgAEUAbQBpAHMAcwBpAG8AbgAgAEkAbgB0AGUAbgBzAGkAdABpAGUAcwAgAGYAbwByACAATQBhAHQAZQByAGkAYQBsACAASQBuAHAAdQB0AHMAIAB0AG8AIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAQQBnAHIAaQBjAHUAbAB0AHUAcgBlACwAIABGAGkAcwBoAGUAcgBpAGUAcwAgAGEAbgBkACAARgBvAHIAZQBzAHQAcgB5AC4AIABWAGUAcgBzAGkAbwBuACAANAA4AC4AIABkAG8AaQAgADEAMAAuADUAMgA4ADEALwB6AGUAbgBvAGQAbwAuADEAOQA2ADUANgA1ADgAMABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEQAYQBpAHIAeQBjAGEAdAB0AGwAZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AFwAIgAsACAAXAAiAFMAbwB1AHIAYwBlACAAcgBlAGcAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAaQByAHkAIABjAG8AdwBzAFwAIgAsACAAXAAiAFYASQBDAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBQAGkAZwBzACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUABpAGcAcwBfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAaQBnAHMAXAAiACwAIABcACIAQQB1AHMAdAByAGEAbABpAGEAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUwBoAGUAZQBwAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBTAGgAZQBlAHAAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFMAaABlAGUAcAAgAHAAcgBvAGQAdQBjAHQAcwAgAGYAbwByACAAcwBjAG8AcABlACAAMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFMAaABlAGUAcABfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBTAGgAZQBlAHAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFMAaABlAGUAcABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBMAGkAZgBlAGMAeQBjAGwAZQBzAC4AIAAoADIAMAAyADYAKQAuACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAEcAYQBzACAARQBtAGkAcwBzAGkAbwBuACAASQBuAHQAZQBuAHMAaQB0AGkAZQBzACAAZgBvAHIAIABNAGEAdABlAHIAaQBhAGwAIABJAG4AcAB1AHQAcwAgAHQAbwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABBAGcAcgBpAGMAdQBsAHQAdQByAGUALAAgAEYAaQBzAGgAZQByAGkAZQBzACAAYQBuAGQAIABGAG8AcgBlAHMAdAByAHkALgAgAFYAZQByAHMAaQBvAG4AIAA0ADgALgAgAGQAbwBpACAAMQAwAC4ANQAyADgAMQAvAHoAZQBuAG8AZABvAC4AMQA5ADYANQA2ADUAOAAwAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUwBoAGUAZQBwAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAaABlAGUAcAAsACAAZgBvAHIAIABtAHUAdAB0AG8AbgBcACIALAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAaABlAGUAcAAsACAAZgBvAHIAIABwAHIAaQBtAGUAIABsAGEAbQBiAFwAIgAsACAAXAAiAE4AUwBXAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAUQBMAEQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBTAEEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFYASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAVwBBAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFIATwBXACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwAKQAgACsAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACAALQAgADEAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAVABhAGIAbABlAEgAZQBhAGQAZQByAEMAZQBsAGwALABcAG4AIAAgAEMATwBMAFUATQBOACgAVABhAGIAbABlAEgAZQBhAGQAZQByAEMAZQBsAGwAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAHIAYQB5AEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIABBAHIAcgBhAHkARABhAHQAYQAsACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkALAAgAFsAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQBdACwAXABuACAASQBGAEUAUgBSAE8AUgAoAFwAbgAgACAAIAAgACAASQBOAEQARQBYACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFUATgBJAFEAVQBFACgAQQByAHIAYQB5AEQAYQB0AGEAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBXACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABDAE8ATABVAE0ATgAoACkALQBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5ACkALAAgADEALAAgAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALAAgAFwAIgBcACIAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABJAEYAKABJAFMATgBVAE0AQgBFAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkAXABuACAAIAAgACAAKQAsACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQAsACAAMAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAVAB3AG8AQwBvAGwAdQBtAG4AcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIAAoAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlADEAKQAqACgATABvAG8AawB1AHAAQQByAHIAYQB5ADIAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgApACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAKQAsACAAXAAiAFwAIgAsACAAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAKQApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABbAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlAF0ALABcAG4AIAAgACAAIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBmAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBmAEYAYQBsAHMAZQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABDAGUAbABsACwAIABEAGUAbABpAG0AaQB0AGUAcgAsACAAWwBDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQBdACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyAF0ALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSAFgATQBMACgAXABuACAAIAAgACAAIAAgACAAIABcACIAXAB1ADAAMAAzAGMAdABcAHUAMAAwADMAZQBcAHUAMAAwADMAYwBzAFwAdQAwADAAMwBlAFwAIgAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAUwBVAEIAUwBUAEkAVABVAFQARQAoAEMAZQBsAGwALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQAsAFwAIgBcACIAKQAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAZQBsAGkAbQBpAHQAZQByACwAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwBzAFwAdQAwADAAMwBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgACkAIABcAHUAMAAwADIANgBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwAvAHMAXAB1ADAAMAAzAGUAXAB1ADAAMAAzAGMALwB0AFwAdQAwADAAMwBlAFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAC8ALwBzAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAYQB2AGcAVABlAG0AcAAsAGEAdgBnAFIAYQBpAG4ALABmAHIAbwBzAHQARABhAHkAcwAsAGUAbABlAHYALABtAGEAcABfAHAAZQB0ACwAXABuACAAIAAgACAAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkALABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQAsAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABtAGEAeABFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBQAEUAVABBAHIAcgBhAHkALABtAGEAeABQAEUAVABBAHIAcgBhAHkALABcAG4AIAAgACAAIABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBSAGEAaQBuACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AZgByAG8AcwB0AEQAYQB5AHMAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABGAHIAbwBzAHQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AZQBsAGUAdgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AZQBsAGUAdgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAFAARQBUAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AbQBhAHAAXwBwAGUAdAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFAARQBUAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AbQBhAHAAXwBwAGUAdAApACwAXABuACAAIAAgACAAIAAgACAAIABUAEEASwBFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgAYwBsAGkAbQBhAHQAZQBaAG8AbgBlAEEAcgByAGEAeQAsAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAMQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATQBpAG4AQQByAHIAYQB5ACwAIABNAGEAeABBAHIAcgBhAHkALAAgAEkAdABlAG0AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBpAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGEAeABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACwAXABuACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAEkAdABlAG0AQQByAHIAYQB5ACwAIABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABDAHIAaQB0AGUAcgBpAGEAMQAsACAAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkALAAgAFEAdQBhAG4AdABpAHQAeQAsACAAWwBNAHUAbAB0AGkAcABsAGkAZQByAF0ALAAgAFsAQwByAGkAdABlAHIAaQBhADIAXQAsAFsAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AF0ALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAbQB1AGwAdABpAHAAbABpAGUAcgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABNAHUAbAB0AGkAcABsAGkAZQByACkALAAxACwATQB1AGwAdABpAHAAbABpAGUAcgApACwAXABuACAAIAAgACAAcQB1AGEAbgB0AGkAdAB5ACwAIABRAHUAYQBuAHQAaQB0AHkAKgBNAHUAbAB0AGkAcABsAGkAZQByACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAxACkALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMgAsAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwByAGkAdABlAHIAaQBhADIAKQAsADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMgApACkALABcAG4AIAAgACAAIABTAFUATQBQAFIATwBEAFUAQwBUACgAYwByAGkAdABlAHIAaQBhADEAKgBjAHIAaQB0AGUAcgBpAGEAMgAqAHEAdQBhAG4AdABpAHQAeQApAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAXAB1ADAAMAAzAGMAIABTACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAXAB1ADAAMAAzAGUAIABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAIAAvACoAaABlAGwAcABlAHIAOgAgAGUAbgBkACAAZABhAHQAZQAgAGYAbwByACAAYQAgAHIAZQBwAG8AcgB0AGkAbgBnACAAcABlAHIAaQBvAGQAIABzAHQAYQByAHQAaQBuAGcAIABhAHQAIABhACAAZwBpAHYAZQBuACAAZABhAHQAZQAqAC8AXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALAAgAC8AKgBvAG4AbAB5ACAAbgBlAGUAZAAgAHQAbwAgAGwAbwBvAGsAIABiAGEAYwBrACAAMwA2ADUAIABkAGEAeQBzACgAbQBhAHgAIABvAHYAZQByAGwAYQBwACAAdwBpAG4AZABvAHcAKQAqAC8AXABuACAAIAAgACAAIAAgACAAIABBACwAUwAtADMANgA1ACwAXABuACAAIAAgACAAIAAgACAAIAB5AGEALABZAEUAQQBSACgAQQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AGIALABZAEUAQQBSACgARQApACwAIAAvACoAaQBmACAAdABoAGUAIABhAG4AYwBoAG8AcgAgAGYAbwByACAAeQBhACAAZQBuAGQAcwAgAGIAZQBmAG8AcgBlACAAUwAsAGkAdAAgAGMAYQBuAFwAdQAwADAAMgA3AHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAbgBlAHgAdAAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQBcAHUAMAAwADMAYwBTACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGIAIABzAHQAYQByAHQAcwAgAGEAZgB0AGUAcgAgAEUALABpAHQAIABjAGEAbgBcAHUAMAAwADIANwB0ACAAbwB2AGUAcgBsAGEAcAA7ACAAbQBvAHYAZQAgAHQAbwAgAHAAcgBlAHYAaQBvAHUAcwAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQBcAHUAMAAwADMAZQBFACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4ALABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQByAHMALABTAEUAUQBVAEUATgBDAEUAKABuACwAMQAsAGYAaQByAHMAdABZAGUAYQByACwAMQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwAsAEQAQQBUAEUAKAB5AHIAcwAsAG0ALABkACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMALABNAEEAUAAoAHMAdABhAHIAdABzACwAUABlAHIAaQBvAGQARQBuAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAdABhAGcALABJAEYAKABzAHQAYQByAHQAcwA9AFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcACIAIAAoAFQAaABpAHMAIAByAGUAcABvAHIAdABpAG4AZwAgAGMAeQBjAGwAZQApAFwAIgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMAVABlAHgAdAAsAFQARQBYAFQAKABzAHQAYQByAHQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMAVABlAHgAdAAsAFQARQBYAFQAKABlAG4AZABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbgA9ADAALABcACIAXAAiACwASABTAFQAQQBDAEsAKABzAHQAYQByAHQAcwBUAGUAeAB0ACAAXAB1ADAAMAAyADYAIABcACIAIAB0AG8AIABcACIAIABcAHUAMAAwADIANgAgAGUAbgBkAHMAVABlAHgAdAAgAFwAdQAwADAAMgA2ACAAdABhAGcAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlAFwAbgA9AEwAQQBNAEIARABBACgARgB1AG4AYwB0AGkAbwBuACwAIABUAEUAWABUAEIARQBGAE8AUgBFACgARgBPAFIATQBVAEwAQQBUAEUAWABUACgARgB1AG4AYwB0AGkAbwBuACkALAAgAFwAIgAoAFwAIgApACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQAsAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAD0AXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAIAA9ACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgAMQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkAPQBQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQA9AEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQA9AFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAXAB1ADAAMAAzAGUAMAAsACAAMQAsACAAMAApAFwAbgAgACAAIAAgACkAKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBDAG8AbgB2AGUAcgB0AFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAFQAbwBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlACwAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAQQByAHIAYQB5ACwAIABTAHQAYQB0AGUAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlACwAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAFwAbgA9AEwAQQBNAEIARABBACgAVABhAHIAZwBlAHQAQwBlAGwAbAAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABzAGgALAAgAFQARQBYAFQAQQBGAFQARQBSACgAQwBFAEwATAAoAFwAIgBmAGkAbABlAG4AYQBtAGUAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALAAgAFwAIgBdAFwAIgApACwAXABuACAAIAAgACAAYQBkAGQAcgAsACAAQwBFAEwATAAoAFwAIgBhAGQAZAByAGUAcwBzAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAXABuACAAIAAgACAAXAAiACMAXAB1ADAAMAAyADcAXAAiACAAXAB1ADAAMAAyADYAIABzAGgAIABcAHUAMAAwADIANgAgAFwAIgBcAHUAMAAwADIANwAhAFwAIgAgAFwAdQAwADAAMgA2ACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBEAGkAZgBmAGUAcgBlAG4AdABTAGgAZQBlAHQAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcACIAIABcAHUAMAAwADIANgAgAGEAZABkAHIAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADEAXwAyAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAXABuACAAIAAgACAAQwBIAE8ATwBTAEUAQwBPAEwAUwAoAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsACAAMQAsACAAMgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADMAXwA0AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAXABuACAAIAAgACAAQwBIAE8ATwBTAEUAQwBPAEwAUwAoAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsACAAMwAsACAANAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEcAZQB0AE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACwAIABNAE0AUwAsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAXABuACAAIAAgACAAIAAgACAAIABNAEUARABJAEEATgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAE8AVQBOAEQAKABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgADAAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0ASQBOACgAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBBAFgAKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATQBNAFMALAAgAE0ATQBTAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBSAGUAcwB1AGwAdABzAEkAdABlAG0ARgByAG8AbQBFAHEAdQBhAHQAaQBvAG4AVABpAHQAbABlAEEAbgBkAFMAbwB1AHIAYwBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABpAHQAbABlAEMAZQBsAGwALAAgAFMAbwB1AHIAYwBlAEMAZQBsAGwALABcAG4AIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgATABFAEYAVAAoAFMAbwB1AHIAYwBlAEMAZQBsAGwALAAgAEYASQBOAEQAKABcACIALABcACIALAAgAFMAbwB1AHIAYwBlAEMAZQBsAGwAKQAgAC0AMQApACwAIABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAXAAiACwAIABcACIAXAAiACkAIABcAHUAMAAwADIANgAgAFwAIgAgAFwAIgAgAFwAdQAwADAAMgA2ACAAVABpAHQAbABlAEMAZQBsAGwAXABuACkAOwAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAXAB1ADAAMAAzAGUAMAAsACAAMQAsACAAMAApAFwAbgAgACAAIAAgACkAKQA7AFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEMAYQBsAGMAdQBsAGEAdABlAEgAYQByAHYAZQBzAHQASQBuAGQAZQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQwByAG8AcABUAHkAcABlACwAIABDAHIAbwBwAFQAeQBwAGUAQQByAHIAYQB5ACwAIABSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgADEALwAoADEAKwBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAEMAcgBvAHAAVAB5AHAAZQAsACAAQwByAG8AcABUAHkAcABlAEEAcgByAGEAeQAsACAAUgBlAHMAaQBkAHUAZQBDAHIAbwBwAFIAYQB0AGkAbwBBAHIAcgBhAHkAKQApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAASABhAHIAdgBlAHMAdABJAG4AZABlAHgALABcAG4AIAAgACAAIAAoADEALQBIAGEAcgB2AGUAcwB0AEkAbgBkAGUAeAApAC8ASABhAHIAdgBlAHMAdABJAG4AZABlAHgAXABuACkAOwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBGAHIAYQBjAHQAaQBvAG4AUgBlAHMAaQBkAHUAZQBSAGUAbQBvAHYAZQBkAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABvAHQAYQBsAFIAZQBzAGkAZAB1AGUALAAgAEEAbQBvAHUAbgB0AFIAZQBtAG8AdgBlAGQALABcAG4AIAAgACAAIAAoAEEAbQBvAHUAbgB0AFIAZQBtAG8AdgBlAGQAKgAxADAAXgAzACkALwAoAFQAbwB0AGEAbABSAGUAcwBpAGQAdQBlACoAMQAwAF4AMwApAFwAbgApACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAiACwAIgB0AGUAeAB0ACIAOgAiAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4ANQAuADEAOgAgAE8AdABoAGUAcgAgAEwAaQB2AGUAcwB0AG8AYwBrACAALQAgAEUAbgB0AGUAcgBpAGMAIABmAGUAcgBtAGUAbgB0AGEAdABpAG8AbgAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABlAGEAYwBoACAAbwB0AGgAZQByACAAbABpAHYAZQBzAHQAbwBjAGsAIAB0AHkAcABlACAAKABrAGcAIABDAEgANAAvAGgAZQBhAGQALwB5AGUAYQByACkAIAAoAE0AagApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATwB0AGgAZQByACAATABpAHYAZQBzAHQAbwBjAGsAIAAtACAARQBuAHQAZQByAGkAYwAgAGYAZQByAG0AZQBuAHQAYQB0AGkAbwBuACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGUAYQBjAGgAIABvAHQAaABlAHIAIABsAGkAdgBlAHMAdABvAGMAawAgAHQAeQBwAGUAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBqAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABDAEgANAAgAC8AIABoAGUAYQBkACAALwAgAHkAZQBhAHIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADUALgAxAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAyACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AdABoAGUAcgAgAEwAaQB2AGUAcwB0AG8AYwBrACAAVAB5AHAAZQBcACIALAAgAFwAIgBNAGoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBmAGYAYQBsAG8AXAAiACwAIAA2ADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBvAGEAdABzAFwAIgAsACAANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGUAZQByAFwAIgAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAYQBtAGUAbABzAFwAIgAsACAANAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbABwAGEAYwBhAHMAXAAiACwAIAA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHMAZQBzAFwAIgAsACAAMQA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AdQBsAGUAcwAvAGEAcwBzAGUAcwBcACIALAAgADEAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AdQBzAC8AbwBzAHQAcgBpAGMAaABlAHMAXAAiACwAIAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBQAHIAbwBkAHUAYwBlAGQAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4ANQAuADIAOgAgAE8AdABoAGUAcgAgAEwAaQB2AGUAcwB0AG8AYwBrACAALQAgAFYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZABzACAAcAByAG8AZAB1AGMAZQBkACAAYgB5ACAAZQBhAGMAaAAgAG8AdABoAGUAcgAgAGwAaQB2AGUAcwB0AG8AYwBrACAAdAB5AHAAZQAgACgAawBnACAAVgBTAC8AaABlAGEAZAAvAGQAYQB5ACkAIAAoAFYAUwBqACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBQAHIAbwBkAHUAYwBlAGQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE8AdABoAGUAcgAgAEwAaQB2AGUAcwB0AG8AYwBrACAALQAgAFYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZABzACAAcAByAG8AZAB1AGMAZQBkACAAYgB5ACAAZQBhAGMAaAAgAG8AdABoAGUAcgAgAGwAaQB2AGUAcwB0AG8AYwBrACAAdAB5AHAAZQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBQAHIAbwBkAHUAYwBlAGQAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAUwBqAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFAAcgBvAGQAdQBjAGUAZABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAFYAUwAgAC8AIABoAGUAYQBkACAALwAgAGQAYQB5AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFAAcgBvAGQAdQBjAGUAZABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADUALgAyAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFAAcgBvAGQAdQBjAGUAZABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBQAHIAbwBkAHUAYwBlAGQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOQAsACAAMgAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAHQAaABlAHIAIABMAGkAdgBlAHMAdABvAGMAawAgAFQAeQBwAGUAXAAiACwAIABcACIAVgBTAGoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBmAGYAYQBsAG8AXAAiACwAIAAyAC4ANwAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEcAbwBhAHQAcwBcACIALAAgADAALgAzADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGUAcgBcACIALAAgADAALgA5ADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBhAG0AZQBsAHMAXAAiACwAIAAyAC4ANwAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbABwAGEAYwBhAHMAXAAiACwAIAAwAC4AMwA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHMAZQBzAFwAIgAsACAAMgAuADcAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAHUAbABlAHMALwBhAHMAcwBlAHMAXAAiACwAIAAwAC4AOQAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAbQB1AHMALwBvAHMAdAByAGkAYwBoAGUAcwBcACIALAAgADAALgAzADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGUAZABcAG4AVABhAGIAbABlACAAQQAuADEALgA1AC4AMwA6ACAATwB0AGgAZQByACAATABpAHYAZQBzAHQAbwBjAGsAIAAtACAATgBpAHQAcgBvAGcAZQBuACAAZQB4AGMAcgBlAHQAZQBkACAAcABlAHIAIABsAGkAdgBlAHMAdABvAGMAawAgAHQAeQBwAGUAIAAoAGsAZwAgAE4AMgBPAC8AaABlAGEAZAAvAHkAZQBhAHIAKQAgACgATgBFAGoAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGUAZABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATwB0AGgAZQByACAATABpAHYAZQBzAHQAbwBjAGsAIAAtACAATgBpAHQAcgBvAGcAZQBuACAAZQB4AGMAcgBlAHQAZQBkACAAcABlAHIAIABsAGkAdgBlAHMAdABvAGMAawAgAHQAeQBwAGUAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAZQBkAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAEUAagBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABlAGQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAgAC8AIABoAGUAYQBkACAALwAgAHkAZQBhAHIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAZQBkAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4ANQAuADMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAZQBkAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGUAZABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAyACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AdABoAGUAcgAgAEwAaQB2AGUAcwB0AG8AYwBrACAAVAB5AHAAZQBcACIALAAgAFwAIgBOAEUAagBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgB1AGYAZgBhAGwAbwBcACIALAAgADMAOQAuADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBvAGEAdABzAFwAIgAsACAANwAuADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGUAcgBcACIALAAgADEAMwAuADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBhAG0AZQBsAHMAXAAiACwAIAAzADkALgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbABwAGEAYwBhAHMAXAAiACwAIAA3AC4AMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAG8AcgBzAGUAcwBcACIALAAgADMAOQAuADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQB1AGwAZQBzAC8AYQBzAHMAZQBzAFwAIgAsACAAMQAzAC4AMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AdQBzAC8AbwBzAHQAcgBpAGMAaABlAHMAXAAiACwAIAA3AC4AMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBBAHYAZQByAGEAZwBlAEwAaQB2AGUAdwBlAGkAZwBoAHQAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4ANQAuADQAOgAgAE8AdABoAGUAcgAgAEwAaQB2AGUAcwB0AG8AYwBrACAALQAgAEEAdgBlAHIAYQBnAGUAIABMAGkAdgBlAHcAZQBpAGcAaAB0AHMAIAAoAFcAYwBvACkAIAAoAGsAZwApACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAEEAdgBlAHIAYQBnAGUATABpAHYAZQB3AGUAaQBnAGgAdABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATwB0AGgAZQByACAATABpAHYAZQBzAHQAbwBjAGsAIAAtACAAQQB2AGUAcgBhAGcAZQAgAEwAaQB2AGUAdwBlAGkAZwBoAHQAcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAEEAdgBlAHIAYQBnAGUATABpAHYAZQB3AGUAaQBnAGgAdABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVwBjAG8AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBBAHYAZQByAGEAZwBlAEwAaQB2AGUAdwBlAGkAZwBoAHQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBBAHYAZQByAGEAZwBlAEwAaQB2AGUAdwBlAGkAZwBoAHQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA1AC4ANABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAEEAdgBlAHIAYQBnAGUATABpAHYAZQB3AGUAaQBnAGgAdABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAEEAdgBlAHIAYQBnAGUATABpAHYAZQB3AGUAaQBnAGgAdABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADEALAAgADMALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAATABpAHYAZQBzAHQAbwBjAGsAIABUAHkAcABlACAAagBcACIALAAgAFwAIgBBAHYAZQByAGEAZwBlACAATABpAHYAZQB3AGUAaQBnAGgAdABcACIALAAgAFwAIgBBAHYAZQByAGEAZwBlACAATABpAHYAZQB3AGUAaQBnAGgAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgB1AGYAZgBhAGwAbwBcACIALAAgADMAMwA2ACwAIABcACIALQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBvAGEAdABzAFwAIgAsACAAMwAzACwAIABcACIAMgA4AGsAZwAgAC0AIABsAG8AdwAgAHAAcgBvAGQAdQBjAHQAaQB2AGkAdAB5ACAAcwB5AHMAdABlAG0AcwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBvAGEAdABzAFwAIgAsACAAMwAzACwAIABcACIANQAwAGsAZwAgAC0AIABoAGkAZwBoACAAcAByAG8AZAB1AGMAdABpAHYAaQB0AHkAIABzAHkAcwB0AGUAbQBzAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGUAZQByAFwAIgAsACAAMQAyADAALAAgADEAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAYQBtAGUAbABzAFwAIgAsACAAMgAxADcALAAgADUANwAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbABwAGEAYwBhAHMAXAAiACwAIABcACIALQBcACIALAAgADYANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAG8AcgBzAGUAcwBcACIALAAgADMANwA3ACwAIAA1ADUAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAHUAbABlAHMALwBhAHMAcwBlAHMAXAAiACwAIAAxADMAMAAsACAAMgA0ADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBtAHUAcwAvAG8AcwB0AHIAaQBjAGgAZQBzAFwAIgAsACAAMQAyADAALAAgADEAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBmAGUAcgBlAG4AYwBlAFwAIgAsACAAXAAiAEkAUABDAEMAIAAyADAAMQA5ACAAVABhAGIAbABlACAAMQAwAEEALgA1ACAAWwAyAF0AXAAiACwAIABcACIASQBQAEMAQwAgADIAMAAxADkAIABUAGEAYgBsAGUAIAAxADAALgAxADAAIABbADIAXQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ARgByAGEAYwB0AGkAbwBuAFcAYQBzAHQAZQBJAG4ATQBNAFMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4ANQAuADUAOgAgAE8AdABoAGUAcgAgAEwAaQB2AGUAcwB0AG8AYwBrACAALQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAHcAYQBzAHQAZQAgAGkAbgAgAGUAYQBjAGgAIABtAGEAbgB1AHIAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABzAHkAcwB0AGUAbQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0ATQBTAG0AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ARgByAGEAYwB0AGkAbwBuAFcAYQBzAHQAZQBJAG4ATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE8AdABoAGUAcgAgAEwAaQB2AGUAcwB0AG8AYwBrACAALQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAHcAYQBzAHQAZQAgAGkAbgAgAGUAYQBjAGgAIABtAGEAbgB1AHIAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABzAHkAcwB0AGUAbQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAEYAcgBhAGMAdABpAG8AbgBXAGEAcwB0AGUASQBuAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE0AUwBtAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ARgByAGEAYwB0AGkAbwBuAFcAYQBzAHQAZQBJAG4ATQBNAFMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBGAHIAYQBjAHQAaQBvAG4AVwBhAHMAdABlAEkAbgBNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADUALgA1AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ARgByAGEAYwB0AGkAbwBuAFcAYQBzAHQAZQBJAG4ATQBNAFMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBGAHIAYQBjAHQAaQBvAG4AVwBhAHMAdABlAEkAbgBNAE0AUwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAzACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQBcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBDAFQAXAAiACwAIAAgADkAOQAuADYANgAsACAAIAAwAC4AMwA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AUwBXAFwAIgAsACAAIAA5ADkALgA2ADYALAAgACAAMAAuADMANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAFQAXAAiACwAIAAgADkAOQAuADYANgAsACAAIAAwAC4AMwA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEATABEAFwAIgAsACAAIAA5ADkALgA2ADYALAAgACAAMAAuADMANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAEEAXAAiACwAIAAgADkAOQAuADYANgAsACAAIAAwAC4AMwA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAQQBTAFwAIgAsACAAIAA5ADkALgA2ADYALAAgACAAMAAuADMANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEkAQwBcACIALAAgACAAOQA5AC4ANgA2ACwAIAAgADAALgAzADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBBAFwAIgAsACAAIAA5ADkALgA2ADYALAAgACAAMAAuADMANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAEMAbwBuAHYAZQByAHMAaQBvAG4ARgBhAGMAdABvAHIAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4ANQAuADYAOgAgAE8AdABoAGUAcgAgAEwAaQB2AGUAcwB0AG8AYwBrACAALQAgAE0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABwAGUAcgAgAHIAZQBnAGkAbwBuACAAKABmAHIAYQBjAHQAaQBvAG4AKQAgACgATQBDAEYAaQBtACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAE0AZQB0AGgAYQBuAGUAQwBvAG4AdgBlAHIAcwBpAG8AbgBGAGEAYwB0AG8AcgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATwB0AGgAZQByACAATABpAHYAZQBzAHQAbwBjAGsAIAAtACAATQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHAAZQByACAAcgBlAGcAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAEMAbwBuAHYAZQByAHMAaQBvAG4ARgBhAGMAdABvAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AQwBGAGkAbQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAE0AZQB0AGgAYQBuAGUAQwBvAG4AdgBlAHIAcwBpAG8AbgBGAGEAYwB0AG8AcgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAE0AZQB0AGgAYQBuAGUAQwBvAG4AdgBlAHIAcwBpAG8AbgBGAGEAYwB0AG8AcgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADUALgA2AFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATQBlAHQAaABhAG4AZQBDAG8AbgB2AGUAcgBzAGkAbwBuAEYAYQBjAHQAbwByAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATQBlAHQAaABhAG4AZQBDAG8AbgB2AGUAcgBzAGkAbwBuAEYAYQBjAHQAbwByAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB0AGEAdABlAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXAAiACwAIABcACIAVQBuAGMAbwB2AGUAcgBlAGQAIABBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAEMAVABcACIALAAgACAAMAAuADAAMAA0ADcALAAgACAAMAAuADcAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAFMAVwBcACIALAAgACAAMAAuADAAMAA0ADcALAAgACAAMAAuADcANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAFQAXAAiACwAIAAgADAALgAwADAANAA3ACwAIAAgADAALgA4ADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUQBMAEQAXAAiACwAIAAgADAALgAwADAANAA3ACwAIAAgADAALgA3ADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBAFwAIgAsACAAIAAwAC4AMAAwADQANwAsACAAIAAwAC4ANwA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAQQBTAFwAIgAsACAAIAAwAC4AMAAwADQANwAsACAAIAAwAC4ANwAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYASQBDAFwAIgAsACAAIAAwAC4AMAAwADQANwAsACAAIAAwAC4ANwA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAQQBcACIALAAgACAAMAAuADAAMAA0ADcALAAgACAAMAAuADcANgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADUALgBYADoAIABPAHQAaABlAHIAIABMAGkAdgBlAHMAdABvAGMAawAgAC0AIABNAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIABwAG8AdABlAG4AdABpAGEAbAAgACgAbQAzACAAQwBIADQAIAAvACAAawBnACAAVgBTACkAIAAoAEIATwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBPAHQAaABlAHIAIABMAGkAdgBlAHMAdABvAGMAawAgAC0AIABNAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIABwAG8AdABlAG4AdABpAGEAbABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEIATwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBtADMAIABDAEgANAAgAC8AIABrAGcAIABWAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4ANQAuAFgAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBOACAAUwBPAFUAUgBDAEUAOgAgAFQAaABlAHIAZQAgAHcAZQByAGUAIABuAG8AIAB2AGEAbAB1AGUAcwAgAGkAbgAgAFYARQBFAFIARwAgAHMAbwAgAHQAaABpAHMAIABkAGEAdABhACAAaABhAHMAIABiAGUAZQBuACAAZwBlAG4AZQByAGEAdABlAGQAIABiAHkAIAB1AHMAaQBuAGcAIABkAG8AYwB1AG0AZQBuAHQAZQBkACAAQgBPACAAdgBhAGwAdQBlAHMAIABmAHIAbwBtACAAbwB0AGgAZQByACAAbABpAHYAZQBzAHQAbwBjAGsAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAATABpAHYAZQBzAHQAbwBjAGsAIABUAHkAcABlAFwAIgAsACAAXAAiAEIATwBcACIALAAgAFwAIgBUAGEAawBlAG4AIABmAHIAbwBtAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAHUAZgBmAGEAbABvAFwAIgAsACAAMAAuADEAOQAsACAAXAAiAEYAZQBlAGQAbABvAHQALAAgAFAAYQBzAHQAdQByAGUAIABiAGUAZQBmAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAG8AYQB0AHMAXAAiACwAIAAwAC4AMgA0ACwAIABcACIAUwBoAGUAZQBwAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGUAZQByAFwAIgAsACAAMAAuADIANAAsACAAXAAiAFMAaABlAGUAcABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBhAG0AZQBsAHMAXAAiACwAIAAwAC4AMgA0ACwAIABcACIAUwBoAGUAZQBwAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGwAcABhAGMAYQBzAFwAIgAsACAAMAAuADIANAAsACAAXAAiAFMAaABlAGUAcABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABvAHIAcwBlAHMAXAAiACwAIAAwAC4AMQA5ACwAIABcACIARgBlAGUAZABsAG8AdAAsACAAUABhAHMAdAB1AHIAZQAgAGIAZQBlAGYAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AdQBsAGUAcwAvAGEAcwBzAGUAcwBcACIALAAgADAALgAyADQALAAgAFwAIgBTAGgAZQBlAHAAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAbQB1AHMALwBvAHMAdAByAGkAYwBoAGUAcwBcACIALAAgADAALgAzADYALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAALQAgAG0AZQBhAHQAIABjAGgAaQBjAGsAZQBuAHMAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABuAGkAdAByAG8AZwBlAG4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABmAHIAbwBtACAAdQByAGkAbgBlACAAYQBuAGQAIABmAGEAZQBjAGUAcwAgAGQAZQBwAG8AcwBpAHQAZQBkACAAbwBuACAAcABhAHMAdAB1AHIAZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG4AaQB0AHIAbwBnAGUAbgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGYAcgBvAG0AIAB1AHIAaQBuAGUAIABhAG4AZAAgAGYAYQBlAGMAZQBzACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMARwBBAFMATQBzAG8AaQBsAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4ASAAzAC0ATgAgACsAIABOAE8AeAAtAE4AKQAvAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4ANwAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMgAxACkAOwBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8ATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADQALgA3ADoAIABNAGEAbgB1AHIAZQAgAE0AYQBuAGEAZwBlAG0AZQBuAHQAIAAtACAATwB0AGgAZQByACAATABpAHYAZQBzAHQAbwBjAGsAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADQALgA3AC4AMQAuADEAIABNAGUAdABoAG8AZAAgADEAIAAtACAATQBhAG4AdQByAGUAIABNAGUAdABoAGEAbgBlACAATwB0AGgAZQByACAATABpAHYAZQBzAHQAbwBjAGsAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAFwAbgBUAG8AdABhAGwAIABhAG4AbgB1AGEAbAAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgByAG8AbQAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAG8AZgAgAG8AdABoAGUAcgAgAGwAaQB2AGUAcwB0AG8AYwBrAFwAbgBFAF8AQwBIADQAXABuAHQAIABDAEgANABcAG4ARQBfAHsAQwBIADQAfQA9AFwAXABzAHUAbQBfAGoAXABcAHMAdQBtAF8AbQAoAE4AXwBqAFwAXAB0AGkAbQBlAHMAIABNAF8AagBtAFwAXAB0AGkAbQBlAHMAIAAzADYANQApAFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAbgBOAF8AagAgAD0AIABhAHYAZQByAGEAZwBlACAAYQBuAG4AdQBhAGwAIABuAHUAbQBiAGUAcgAgAG8AZgAgAGwAaQB2AGUAcwB0AG8AYwBrACAAcABlAHIAIABsAGkAdgBlAHMAdABvAGMAawAgAHQAeQBwAGUAIABqACAAKABoAGUAYQBkACkAXABuAE0AXwBqAG0AIAA9ACAAYQBuAG4AdQBhAGwAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABtAGEAbgB1AHIAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIAAoAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGEAbgB1AHIAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABOAF8AagAsACAATQBfAGoAbQAsAFwAbgAgACAAIAAgAFMAVQBNACgATgBfAGoAIAAqACAATQBfAGoAbQAgACoAIAAzADYANQApACAAKgAgADEAMAAgAF4AIAAtADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAG8AdABhAGwAIABhAG4AbgB1AGEAbAAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgByAG8AbQAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAG8AZgAgAG8AdABoAGUAcgAgAGwAaQB2AGUAcwB0AG8AYwBrAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AQwBIADQAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBIADQAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADcALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAxACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AewBDAEgANAB9AD0AXABcAHMAdQBtAFwAXABuAG8AbABpAG0AaQB0AHMAXwBqAFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AbQAoAE4AXwBqAFwAXAB0AGkAbQBlAHMAIABNAF8AagBtAFwAXAB0AGkAbQBlAHMAIAAzADYANQApAFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AXwBqAFwAIgAsACAAXAAiAGEAdgBlAHIAYQBnAGUAIABhAG4AbgB1AGEAbAAgAG4AdQBtAGIAZQByACAAbwBmACAAbABpAHYAZQBzAHQAbwBjAGsAIABwAGUAcgAgAGwAaQB2AGUAcwB0AG8AYwBrACAAdAB5AHAAZQAgAGoAXAAiACwAIABcACIAaABlAGEAZABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AXwBqAG0AXAAiACwAIABcACIAYQBuAG4AdQBhAGwAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABtAGEAbgB1AHIAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAXAAiACwAIABcACIAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAA0AC4ANwAuADEALgAxACwAIAAoADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAagBcACIALAAgAFwAIgBsAGkAdgBlAHMAdABvAGMAawAgAHQAeQBwAGUAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBtAFwAIgAsACAAXAAiAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAHMAeQBzAHQAZQBtAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAxAF8AXwAyAF8AQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABcAG4AQQBuAG4AdQBhAGwAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABtAGEAbgB1AHIAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAXABuAE0AXwBqAG0AXABuAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAbgBNAF8AagBtAD0AVgBTAF8AagBcAFwAdABpAG0AZQBzACAAQgBfAE8AXABcAHQAaQBtAGUAcwAgAE0ATQBTAF8AbQBcAFwAdABpAG0AZQBzACAATQBDAEYAXwBpAG0AXABcAHQAaQBtAGUAcwAgAFwAXAByAGgAbwBcAG4AVgBTAF8AagAgAD0AIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAKABrAGcALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4AQgBfAE8AIAA9ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAcABvAHQAZQBuAHQAaQBhAGwAIAAoAG0AMwAgAEMASAA0AC8AawBnACAAVgBTACkAXABuAE0ATQBTAF8AbQAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIAB3AGEAcwB0AGUAIABpAG4AIABlAGEAYwBoACAAbQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0AXABuAE0AQwBGAF8AaQBtACAAPQAgAG0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIABhAG4AZAAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAHMAeQBzAHQAZQBtAFwAbgByAGgAbwAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAawBnAC8AbQAzACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMQBfAF8AMgBfAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVgBTAF8AagAsACAAQgBfAE8ALAAgAE0ATQBTAF8AbQAsACAATQBDAEYAXwBpAG0ALAAgAHIAaABvACwAXABuACAAIAAgACAAVgBTAF8AagAgACoAIABCAF8ATwAgACoAIABNAE0AUwBfAG0AIAAqACAATQBDAEYAXwBpAG0AIAAqACAAcgBoAG8AXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAxAF8AXwAyAF8AQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBuAG4AdQBhAGwAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABtAGEAbgB1AHIAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADEAXwBfADIAXwBBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGEAbgB1AHIAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAF8AagBtAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAxAF8AXwAyAF8AQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAxAF8AXwAyAF8AQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4ANwAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADIAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMQBfAF8AMgBfAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADEAXwBfADIAXwBBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGEAbgB1AHIAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBfAHsAagBtAH0APQBWAFMAXwBqAFwAXAB0AGkAbQBlAHMAIABCAF8ATwBcAFwAdABpAG0AZQBzACAATQBNAFMAXwBtAFwAXAB0AGkAbQBlAHMAIABNAEMARgBfAHsAaQBtAH0AXABcAHQAaQBtAGUAcwAgAFwAXAByAGgAbwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMQBfAF8AMgBfAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBTAF8AagBcACIALAAgAFwAIgB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAIABwAHIAbwBkAHUAYwB0AGkAbwBuAFwAIgAsACAAXAAiAGsAZwAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAXwBPAFwAIgAsACAAXAAiAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHAAbwB0AGUAbgB0AGkAYQBsAFwAIgAsACAAXAAiAG0AMwAgAEMASAA0AC8AawBnACAAVgBTAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBNAFMAXwBtAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAHcAYQBzAHQAZQAgAGkAbgAgAGUAYQBjAGgAIABtAGEAbgB1AHIAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEMARgBfAGkAbQBcACIALAAgAFwAIgBtAGUAdABoAGEAbgBlACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABzAHQAYQB0AGUAIABhAG4AZAAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAHMAeQBzAHQAZQBtAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAHIAaABvAFwAIgAsACAAXAAiAGQAZQBuAHMAaQB0AHkAIABvAGYAIABtAGUAdABoAGEAbgBlAFwAIgAsACAAXAAiAGsAZwAvAG0AMwBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGkAXAAiACwAIABcACIAcwB0AGEAdABlAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADEAXwBfADIAXwBBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGEAbgB1AHIAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AQQByAGcAdQBtAGUAbgB0AHMAXwBNAGUAdABoAG8AZAAyAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAFMAXwBqAFwAIgAsACAAXAAiAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZAAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AXAAiACwAIABcACIAawBnAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgBfAE8AXAAiACwAIABcACIAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAcABvAHQAZQBuAHQAaQBhAGwAXAAiACwAIABcACIAbQAzACAAQwBIADQALwBrAGcAIABWAFMAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE0AUwBfAG0AXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAdwBhAHMAdABlACAAaQBuACAAZQBhAGMAaAAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAHMAeQBzAHQAZQBtAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQwBGAF8AaQBtAFwAIgAsACAAXAAiAG0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIABhAG4AZAAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAHMAeQBzAHQAZQBtAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAHIAaABvAFwAIgAsACAAXAAiAGQAZQBuAHMAaQB0AHkAIABvAGYAIABtAGUAdABoAGEAbgBlAFwAIgAsACAAXAAiAGsAZwAvAG0AMwBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGkAXAAiACwAIABcACIAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgAsACAAXAAiAGQAZQBnAHIAZQBlAHMAIABDAGUAbABzAGkAdQBzAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBOADIATwBEAGkAcgBlAGMAdAAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ANAAuADcAOgAgAE0AYQBuAHUAcgBlACAATQBhAG4AYQBnAGUAbQBlAG4AdAAgAC0AIABPAHQAaABlAHIAIABMAGkAdgBlAHMAdABvAGMAawBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ANAAuADcALgAxAC4AMwAgAE0AZQB0AGgAbwBkACAAMQAgAC0AIABTAG8AaQBsACAARABpAHIAZQBjAHQAIABOADIATwAgAE8AdABoAGUAcgAgAEwAaQB2AGUAcwB0AG8AYwBrAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMwBfAF8AMQBfAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AUwBvAGkAbABcAG4ARABpAHIAZQBjAHQAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAYQBnAHIAaQBjAHUAbAB0AHUAcgBhAGwAIABzAG8AaQBsAHMAIABmAHIAbwBtACAAZABlAHAAbwBzAGkAdABpAG8AbgAgAG8AZgAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZAB1AG4AZwAgAHQAbwAgAHAAYQBzAHQAdQByAGUAXABuAEUAXwBOADIATwBkAGkAcgBcAG4AdAAgAE4AMgBPAFwAbgBFAF8AewBOADIATwAsAGQAaQByAH0APQBBAEUAXABcAHQAaQBtAGUAcwAgAEUARgBfAHsAUABSAFAAfQBcAFwAdABpAG0AZQBzACAAQwBfAHsATgAyAE8AfQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcAG4AQQBFACAAPQAgAGEAbgBuAHUAYQBsACAAbgBpAHQAcgBvAGcAZQBuACAAZQB4AGMAcgBlAHQAZQBkACAAYgB5ACAAZQBhAGMAaAAgAGwAaQB2AGUAcwB0AG8AYwBrACAAdAB5AHAAZQAgACgAawBnACAATgAvAHkAZQBhAHIAKQBcAG4ARQBGAF8AUABSAFAAIAA9ACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABmAHIAbwBtACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIAB0AG8AIABzAG8AaQBsACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACAAZABlAHAAbwBzAGkAdABlAGQAKQBcAG4AQwBfAE4AMgBPACAAPQAgAGYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMwBfAF8AMQBfAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AUwBvAGkAbABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAEUALAAgAEUARgBfAFAAUgBQACwAIABDAF8ATgAyAE8ALABcAG4AIAAgACAAIABBAEUAIAAqACAARQBGAF8AUABSAFAAIAAqACAAQwBfAE4AMgBPACAAKgAgADEAMAAgAF4AIAAtADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAzAF8AXwAxAF8ARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBTAG8AaQBsAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBEAGkAcgBlAGMAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABhAGcAcgBpAGMAdQBsAHQAdQByAGEAbAAgAHMAbwBpAGwAcwAgAGYAcgBvAG0AIABkAGUAcABvAHMAaQB0AGkAbwBuACAAbwBmACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAdABvACAAcABhAHMAdAB1AHIAZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMwBfAF8AMQBfAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AUwBvAGkAbABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAE4AMgBPAGQAaQByAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAzAF8AXwAxAF8ARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBTAG8AaQBsAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAE4AMgBPAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAzAF8AXwAxAF8ARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBTAG8AaQBsAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgA3AC4AMQAuADMALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAzAF8AXwAxAF8ARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBTAG8AaQBsAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAzAF8AXwAxAF8ARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBTAG8AaQBsAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAHsATgAyAE8ALABkAGkAcgB9AD0AQQBFAFwAXAB0AGkAbQBlAHMAIABFAEYAXwB7AFAAUgBQAH0AXABcAHQAaQBtAGUAcwAgAEMAXwB7AE4AMgBPAH0AXABcAHQAaQBtAGUAcwAgADEAMABeAHsALQAzAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADMAXwBfADEAXwBEAGkAcgBlAGMAdABOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFMAbwBpAGwAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBFAFwAIgAsACAAXAAiAGEAbgBuAHUAYQBsACAAbgBpAHQAcgBvAGcAZQBuACAAZQB4AGMAcgBlAHQAZQBkACAAYgB5ACAAZQBhAGMAaAAgAGwAaQB2AGUAcwB0AG8AYwBrACAAdAB5AHAAZQBcACIALAAgAFwAIgBrAGcAIABOAC8AeQBlAGEAcgBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADQALgA3AC4AMQAuADMALAAgACgAMgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEYAXwBQAFIAUABcACIALAAgAFwAIgBlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGYAcgBvAG0AIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAHQAbwAgAHMAbwBpAGwAXAAiACwAIABcACIAawBnACAATgAyAE8ALQBOAC8AawBnACAATgAgAGQAZQBwAG8AcwBpAHQAZQBkAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBfAE4AMgBPAFwAIgAsACAAXAAiAGYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXAAiACwAIABcACIAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgB6AFwAIgAsACAAXAAiAHcAZQB0ACAAbwByACAAZAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMwBfAF8AMgBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABlAGQAVABvAFAAYQBzAHQAdQByAGUAXABuAEEAbgBuAHUAYQBsACAAbgBpAHQAcgBvAGcAZQBuACAAZQB4AGMAcgBlAHQAZQBkACAAYgB5ACAAbABpAHYAZQBzAHQAbwBjAGsAIAB0AG8AIABwAGEAcwB0AHUAcgBlACwAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAXABuAEEARQBcAG4AawBnACAATgAvAHkAZQBhAHIAXABuAEEARQA9AFwAXABzAHUAbQBfAGoAKABOAF8AagBcAFwAdABpAG0AZQBzACAATgBFAF8AagBcAFwAdABpAG0AZQBzACAAMwA2ADUAKQBcAG4ATgBfAGoAIAA9ACAAbgB1AG0AYgBlAHIAIABvAGYAIABsAGkAdgBlAHMAdABvAGMAawAgAG8AZgAgAGUAYQBjAGgAIABsAGkAdgBlAHMAdABvAGMAawAgAHQAeQBwAGUAIABqACAAKABoAGUAYQBkACkAXABuAE4ARQBfAGoAIAA9ACAAbgBpAHQAcgBvAGcAZQBuACAAZQB4AGMAcgBlAHQAZQBkACAAYgB5ACAAZQBhAGMAaAAgAGwAaQB2AGUAcwB0AG8AYwBrACAAdAB5AHAAZQAgAGoAIAAoAGsAZwAgAE4ALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAzAF8AXwAyAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGUAZABUAG8AUABhAHMAdAB1AHIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABOAF8AagAsACAATgBFAF8AagAsAFwAbgAgACAAIAAgAE4AXwBqACAAKgAgAE4ARQBfAGoAIAAqACAAMwA2ADUAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAzAF8AXwAyAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGUAZABUAG8AUABhAHMAdAB1AHIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBuAG4AdQBhAGwAIABuAGkAdAByAG8AZwBlAG4AIABlAHgAYwByAGUAdABlAGQAIABiAHkAIABsAGkAdgBlAHMAdABvAGMAawAgAHQAbwAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMwBfAF8AMgBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABlAGQAVABvAFAAYQBzAHQAdQByAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEARQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMwBfAF8AMgBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABlAGQAVABvAFAAYQBzAHQAdQByAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOAC8AeQBlAGEAcgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMwBfAF8AMgBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABlAGQAVABvAFAAYQBzAHQAdQByAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADcALgAxAC4AMwAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAyACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADMAXwBfADIAXwBBAG4AbgB1AGEAbABOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAZQBkAFQAbwBQAGEAcwB0AHUAcgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAzAF8AXwAyAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGUAZABUAG8AUABhAHMAdAB1AHIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEARQA9AFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AagAoAE4AXwBqAFwAXAB0AGkAbQBlAHMAIABOAEUAXwBqAFwAXAB0AGkAbQBlAHMAIAAzADYANQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAzAF8AXwAyAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGUAZABUAG8AUABhAHMAdAB1AHIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAF8AagBcACIALAAgAFwAIgBuAHUAbQBiAGUAcgAgAG8AZgAgAGwAaQB2AGUAcwB0AG8AYwBrACAAbwBmACAAZQBhAGMAaAAgAGwAaQB2AGUAcwB0AG8AYwBrACAAdAB5AHAAZQAgAGoAXAAiACwAIABcACIAaABlAGEAZABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARQBfAGoAXAAiACwAIABcACIAbgBpAHQAcgBvAGcAZQBuACAAZQB4AGMAcgBlAHQAZQBkACAAYgB5ACAAZQBhAGMAaAAgAGwAaQB2AGUAcwB0AG8AYwBrACAAdAB5AHAAZQAgAGoAXAAiACwAIABcACIAawBnACAATgAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGoAXAAiACwAIABcACIAbABpAHYAZQBzAHQAbwBjAGsAIAB0AHkAcABlAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ANAAuADcAOgAgAE0AYQBuAHUAcgBlACAATQBhAG4AYQBnAGUAbQBlAG4AdAAgAC0AIABPAHQAaABlAHIAIABMAGkAdgBlAHMAdABvAGMAawBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ANAAuADcALgAxAC4ANQAgAE0AZQB0AGgAbwBkACAAMQAgAC0AIABTAG8AaQBsACAAQQB0AG0AbwBzAHAAaABlAHIAaQBjACAARABlAHAAbwBzAGkAdABpAG8AbgAgAE4AMgBPACAATwB0AGgAZQByACAATABpAHYAZQBzAHQAbwBjAGsAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA1AF8AXwAxAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAFwAbgBBAHQAbQBvAHMAcABoAGUAcgBpAGMAIABkAGUAcABvAHMAaQB0AGkAbwBuACAAZQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlAFwAbgBFAF8ATgAyAE8AYQBkAFwAbgB0ACAATgAyAE8AXABuAEUAXwB7AE4AMgBPACwAYQBkAH0APQBNAF8AewB2AG8AbAB9AFwAXAB0AGkAbQBlAHMAIABFAEYAXwB7AE4AMgBPAH0AXABcAHQAaQBtAGUAcwAgAEMAXwB7AE4AMgBPAH0AXABcAHQAaQBtAGUAcwAgADEAMABeAHsALQAzAH0AXABuAE0AXwB2AG8AbAAgAD0AIABtAGEAcwBzACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAZgByAG8AbQAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZgBhAGUAYwBlAHMAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUAIAAoAGsAZwAgAE4AKQBcAG4ARQBGAF8ATgAyAE8AIAA9ACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGEAdABtAG8AcwBwAGgAZQByAGkAYwAgAGQAZQBwAG8AcwBpAHQAaQBvAG4AIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQBcAG4AQwBfAE4AMgBPACAAPQAgAGYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANQBfAF8AMQBfAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AUABhAHMAdAB1AHIAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAF8AdgBvAGwALAAgAEUARgBfAE4AMgBPACwAIABDAF8ATgAyAE8ALABcAG4AIAAgACAAIABNAF8AdgBvAGwAIAAqACAARQBGAF8ATgAyAE8AIAAqACAAQwBfAE4AMgBPACAAKgAgADEAMAAgAF4AIAAtADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA1AF8AXwAxAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHQAbQBvAHMAcABoAGUAcgBpAGMAIABkAGUAcABvAHMAaQB0AGkAbwBuACAAZQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA1AF8AXwAxAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8ATgAyAE8AYQBkAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA1AF8AXwAxAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAE4AMgBPAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA1AF8AXwAxAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgA3AC4AMQAuADUALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA1AF8AXwAxAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA1AF8AXwAxAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAHsATgAyAE8ALABhAGQAfQA9AE0AXwB7AHYAbwBsAH0AXABcAHQAaQBtAGUAcwAgAEUARgBfAHsATgAyAE8AfQBcAFwAdABpAG0AZQBzACAAQwBfAHsATgAyAE8AfQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANQBfAF8AMQBfAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AUABhAHMAdAB1AHIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAF8AdgBvAGwAXAAiACwAIABcACIAbQBhAHMAcwAgAG8AZgAgAG4AaQB0AHIAbwBnAGUAbgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGYAcgBvAG0AIAB1AHIAaQBuAGUAIABhAG4AZAAgAGYAYQBlAGMAZQBzACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAGsAZwAgAE4AXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAA0AC4ANwAuADEALgA1ACwAIAAoADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAF8ATgAyAE8AXAAiACwAIABcACIAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGEAdABtAG8AcwBwAGgAZQByAGkAYwAgAGQAZQBwAG8AcwBpAHQAaQBvAG4AXAAiACwAIABcACIAawBnACAATgAyAE8ALQBOAC8AawBnACAATgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAXwBOADIATwBcACIALAAgAFwAIgBmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAagBcACIALAAgAFwAIgBwAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBpAFwAIgAsACAAXAAiAGkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAHIAXAAiACwAIABcACIAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBWAG8AbABhAHQAaQBsAGkAcwBlAGQARgByAG8AbQBQAGEAcwB0AHUAcgBlAFwAbgBNAGEAcwBzACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAZgByAG8AbQAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZgBhAGUAYwBlAHMAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUAXABuAE0AXwB2AG8AbABcAG4AawBnACAATgBcAG4ATQBfAHsAdgBvAGwAfQA9AEEARQBcAFwAdABpAG0AZQBzACAARgByAGEAYwBHAEEAUwBNAHMAbwBpAGwAXABuAEEARQAgAD0AIABhAG4AbgB1AGEAbAAgAG4AaQB0AHIAbwBnAGUAbgAgAGUAeABjAHIAZQB0AGUAZAAgAGIAeQAgAGUAYQBjAGgAIABsAGkAdgBlAHMAdABvAGMAawAgAHQAeQBwAGUAIAAoAGsAZwAgAE4ALwB5AGUAYQByACkAXABuAEYAcgBhAGMARwBBAFMATQBzAG8AaQBsACAAPQAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG4AaQB0AHIAbwBnAGUAbgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGYAcgBvAG0AIAB1AHIAaQBuAGUAIABhAG4AZAAgAGYAYQBlAGMAZQBzACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlACAAKAAoAGsAZwAgAE4ASAAzAC0ATgAgACsAIABOAE8AeAAtAE4AKQAvAGsAZwAgAE4AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA1AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAFYAbwBsAGEAdABpAGwAaQBzAGUAZABGAHIAbwBtAFAAYQBzAHQAdQByAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQBFACwAIABGAHIAYQBjAEcAQQBTAE0AcwBvAGkAbAAsAFwAbgAgACAAIAAgAEEARQAgACoAIABGAHIAYQBjAEcAQQBTAE0AcwBvAGkAbABcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADUAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0AUABhAHMAdAB1AHIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAHMAcwAgAG8AZgAgAG4AaQB0AHIAbwBnAGUAbgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGYAcgBvAG0AIAB1AHIAaQBuAGUAIABhAG4AZAAgAGYAYQBlAGMAZQBzACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA1AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAFYAbwBsAGEAdABpAGwAaQBzAGUAZABGAHIAbwBtAFAAYQBzAHQAdQByAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AXwB2AG8AbABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBWAG8AbABhAHQAaQBsAGkAcwBlAGQARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBWAG8AbABhAHQAaQBsAGkAcwBlAGQARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgA3AC4AMQAuADUALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMgApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA1AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAFYAbwBsAGEAdABpAGwAaQBzAGUAZABGAHIAbwBtAFAAYQBzAHQAdQByAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADUAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0AUABhAHMAdAB1AHIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AXwB7AHYAbwBsAH0APQBBAEUAXABcAHQAaQBtAGUAcwAgAEYAcgBhAGMARwBBAFMATQBzAG8AaQBsAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA1AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAFYAbwBsAGEAdABpAGwAaQBzAGUAZABGAHIAbwBtAFAAYQBzAHQAdQByAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBFAFwAIgAsACAAXAAiAGEAbgBuAHUAYQBsACAAbgBpAHQAcgBvAGcAZQBuACAAZQB4AGMAcgBlAHQAZQBkACAAYgB5ACAAZQBhAGMAaAAgAGwAaQB2AGUAcwB0AG8AYwBrACAAdAB5AHAAZQBcACIALAAgAFwAIgBrAGcAIABOAC8AeQBlAGEAcgBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAYgB5ACAANAAuADcALgAxAC4AMwAsACAAKAAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAcgBhAGMARwBBAFMATQBzAG8AaQBsAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG4AaQB0AHIAbwBnAGUAbgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGYAcgBvAG0AIAB1AHIAaQBuAGUAIABhAG4AZAAgAGYAYQBlAGMAZQBzACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiACgAawBnACAATgBIADMALQBOACAAKwAgAE4ATwB4AC0ATgApAC8AawBnACAATgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8ATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA0AC4ANwA6ACAATQBhAG4AdQByAGUAIABNAGEAbgBhAGcAZQBtAGUAbgB0ACAALQAgAE8AdABoAGUAcgAgAEwAaQB2AGUAcwB0AG8AYwBrAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA0AC4ANwAuADEALgA3ACAATQBlAHQAaABvAGQAIAAxACAALQAgAFMAbwBpAGwAIABMAGUAYQBjAGgAaQBuAGcAIABBAG4AZAAgAFIAdQBuAG8AZgBmACAATgAyAE8AIABPAHQAaABlAHIAIABMAGkAdgBlAHMAdABvAGMAawBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADcAXwBfADEAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAFwAbgBMAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmACAAZQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAdQByAGkAbgBlACAAYQBuAGQAIABkAHUAbgBnACAAZABlAHAAbwBzAGkAdABlAGQAIABvAG4AIABwAGEAcwB0AHUAcgBlAFwAbgBFAF8ATgAyAE8AbABlAGEAYwBoAFwAbgB0ACAATgAyAE8AXABuAEUAXwB7AE4AMgBPACwAbABlAGEAYwBoAH0APQBNAF8AewBsAGUAYQBjAGgAfQBcAFwAdABpAG0AZQBzACAARQBGAF8AewBsAGUAYQBjAGgAfQBcAFwAdABpAG0AZQBzACAAQwBfAHsATgAyAE8AfQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcAG4ATQBfAGwAZQBhAGMAaAAgAD0AIABtAGEAcwBzACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAbABvAHMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoAGsAZwAgAE4AKQBcAG4ARQBGAF8AbABlAGEAYwBoACAAPQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACkAXABuAEMAXwBOADIATwAgAD0AIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADcAXwBfADEAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AXwBsAGUAYQBjAGgALAAgAEUARgBfAGwAZQBhAGMAaAAsACAAQwBfAE4AMgBPACwAXABuACAAIAAgACAATQBfAGwAZQBhAGMAaAAgACoAIABFAEYAXwBsAGUAYQBjAGgAIAAqACAAQwBfAE4AMgBPACAAKgAgADEAMAAgAF4AIAAtADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA3AF8AXwAxAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AUABhAHMAdAB1AHIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgAgAGUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZAB1AG4AZwAgAGQAZQBwAG8AcwBpAHQAZQBkACAAbwBuACAAcABhAHMAdAB1AHIAZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANwBfAF8AMQBfAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFAAYQBzAHQAdQByAGUAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwBOADIATwBsAGUAYQBjAGgAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADcAXwBfADEAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAE4AMgBPAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA3AF8AXwAxAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AUABhAHMAdAB1AHIAZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4ANwAuADEALgA3ACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADEAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANwBfAF8AMQBfAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFAAYQBzAHQAdQByAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADcAXwBfADEAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAHsATgAyAE8ALABsAGUAYQBjAGgAfQA9AE0AXwB7AGwAZQBhAGMAaAB9AFwAXAB0AGkAbQBlAHMAIABFAEYAXwB7AGwAZQBhAGMAaAB9AFwAXAB0AGkAbQBlAHMAIABDAF8AewBOADIATwB9AFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA3AF8AXwAxAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AUABhAHMAdAB1AHIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAF8AbABlAGEAYwBoAFwAIgAsACAAXAAiAG0AYQBzAHMAIABvAGYAIABuAGkAdAByAG8AZwBlAG4AIABsAG8AcwB0ACAAdABvACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIALAAgAFwAIgBrAGcAIABOAFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAANAAuADcALgAxAC4ANwAsACAAKAAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBfAGwAZQBhAGMAaABcACIALAAgAFwAIgBlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIALAAgAFwAIgBrAGcAIABOADIATwAtAE4ALwBrAGcAIABOAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBfAE4AMgBPAFwAIgAsACAAXAAiAGYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIAB0AG8AIABtAG8AbABlAGMAdQBsAGEAcgAgAG0AYQBzAHMAXAAiACwAIABcACIAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAFwAbgBNAGEAcwBzACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAbABvAHMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAE0AXwBsAGUAYQBjAGgAXABuAGsAZwAgAE4AXABuAE0AXwB7AGwAZQBhAGMAaAB9AD0AQQBFAFwAXAB0AGkAbQBlAHMAIABGAHIAYQBjAFcAZQB0AFwAXAB0AGkAbQBlAHMAIABGAHIAYQBjAEwARQBBAEMASABcAG4AQQBFACAAPQAgAGEAbgBuAHUAYQBsACAAbgBpAHQAcgBvAGcAZQBuACAAZQB4AGMAcgBlAHQAZQBkACAAYgB5ACAAZQBhAGMAaAAgAGwAaQB2AGUAcwB0AG8AYwBrACAAdAB5AHAAZQAgACgAawBnACAATgAvAHkAZQBhAHIAKQBcAG4ARgByAGEAYwBXAGUAdAAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABuAGkAdAByAG8AZwBlAG4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ARgByAGEAYwBMAEUAQQBDAEgAIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAYQBsAGwAIABuAGkAdAByAG8AZwBlAG4AIAB0AGgAYQB0ACAAaQBzACAAbABvAHMAdAAgAHQAaAByAG8AdQBnAGgAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEEARQAsACAARgByAGEAYwBXAGUAdAAsACAARgByAGEAYwBMAEUAQQBDAEgALABcAG4AIAAgACAAIABBAEUAIAAqACAARgByAGEAYwBXAGUAdAAgACoAIABGAHIAYQBjAEwARQBBAEMASABcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAcwBzACAAbwBmACAAbgBpAHQAcgBvAGcAZQBuACAAbABvAHMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAF8AbABlAGEAYwBoAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA3AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABvAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgA3AC4AMQAuADcALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMgApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA3AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABvAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANwBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAbwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAF8AewBsAGUAYQBjAGgAfQA9AEEARQBcAFwAdABpAG0AZQBzACAARgByAGEAYwBXAGUAdABcAFwAdABpAG0AZQBzACAARgByAGEAYwBMAEUAQQBDAEgAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEARQBcACIALAAgAFwAIgBhAG4AbgB1AGEAbAAgAG4AaQB0AHIAbwBnAGUAbgAgAGUAeABjAHIAZQB0AGUAZAAgAGIAeQAgAGUAYQBjAGgAIABsAGkAdgBlAHMAdABvAGMAawAgAHQAeQBwAGUAXAAiACwAIABcACIAawBnACAATgAvAHkAZQBhAHIAXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGIAeQAgADQALgA3AC4AMQAuADMALAAgACgAMgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAHIAYQBjAFcAZQB0AFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG4AaQB0AHIAbwBnAGUAbgAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAYQBsAGwAIABuAGkAdAByAG8AZwBlAG4AIAB0AGgAYQB0ACAAaQBzACAAbABvAHMAdAAgAHQAaAByAG8AdQBnAGgAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAegBcACIALAAgAFwAIgBsAG8AYwBhAHQAaQBvAG4AIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAagBcACIALAAgAFwAIgBwAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBpAHIAXAAiACwAIABcACIAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AIgB9AF0ALAAiAHAAcgBvAGoAZQBjAHQATgBhAG0AZQBzACIAOgBbACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFYAYQBpAHIAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE8AbgBlAEMAbwBsAHUAbQBuAEEAbgBkAEgAZQBhAGQAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAATgAyAE8ARQBGAEYAcgBvAG0AUAByAG8AZABJAHIAcgBpAGcAYQB0AGkAbwBuAFIAYQBpAG4AZgBhAGwAbAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AQwBvAG4AdgBlAHIAdABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBUAG8AQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADEAXwAyACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAzAF8ANAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVAAiACwAIgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBIAGEAcgB2AGUAcwB0AEkAbgBkAGUAeAAiACwAIgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvACIALAAiAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEMAYQBsAGMAdQBsAGEAdABlAEYAcgBhAGMAdABpAG8AbgBSAGUAcwBpAGQAdQBlAFIAZQBtAG8AdgBlAGQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4ARgBhAGMAdABvAHIAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAEYAYQBjAHQAbwByAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBGAGEAYwB0AG8AcgBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAHMAUAByAG8AZAB1AGMAZQBkAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFAAcgBvAGQAdQBjAGUAZABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAcwBQAHIAbwBkAHUAYwBlAGQAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFAAcgBvAGQAdQBjAGUAZABfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFAAcgBvAGQAdQBjAGUAZABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABzAFAAcgBvAGQAdQBjAGUAZABfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAZQBkAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGUAZABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABlAGQAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGUAZABfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGUAZABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGUAZABfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBBAHYAZQByAGEAZwBlAEwAaQB2AGUAdwBlAGkAZwBoAHQAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBBAHYAZQByAGEAZwBlAEwAaQB2AGUAdwBlAGkAZwBoAHQAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBBAHYAZQByAGEAZwBlAEwAaQB2AGUAdwBlAGkAZwBoAHQAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AQQB2AGUAcgBhAGcAZQBMAGkAdgBlAHcAZQBpAGcAaAB0AF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBBAHYAZQByAGEAZwBlAEwAaQB2AGUAdwBlAGkAZwBoAHQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAEEAdgBlAHIAYQBnAGUATABpAHYAZQB3AGUAaQBnAGgAdABfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBGAHIAYQBjAHQAaQBvAG4AVwBhAHMAdABlAEkAbgBNAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAEYAcgBhAGMAdABpAG8AbgBXAGEAcwB0AGUASQBuAE0ATQBTAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ARgByAGEAYwB0AGkAbwBuAFcAYQBzAHQAZQBJAG4ATQBNAFMAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ARgByAGEAYwB0AGkAbwBuAFcAYQBzAHQAZQBJAG4ATQBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAEYAcgBhAGMAdABpAG8AbgBXAGEAcwB0AGUASQBuAE0ATQBTAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBGAHIAYQBjAHQAaQBvAG4AVwBhAHMAdABlAEkAbgBNAE0AUwBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAEMAbwBuAHYAZQByAHMAaQBvAG4ARgBhAGMAdABvAHIAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAEMAbwBuAHYAZQByAHMAaQBvAG4ARgBhAGMAdABvAHIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAEMAbwBuAHYAZQByAHMAaQBvAG4ARgBhAGMAdABvAHIAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATQBlAHQAaABhAG4AZQBDAG8AbgB2AGUAcgBzAGkAbwBuAEYAYQBjAHQAbwByAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAEMAbwBuAHYAZQByAHMAaQBvAG4ARgBhAGMAdABvAHIAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAE0AZQB0AGgAYQBuAGUAQwBvAG4AdgBlAHIAcwBpAG8AbgBGAGEAYwB0AG8AcgBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ARgByAGEAYwBHAEEAUwBNAFMAbwBpAGwAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAEYAcgBhAGMARwBBAFMATQBTAG8AaQBsAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBGAHIAYQBjAEcAQQBTAE0AUwBvAGkAbABfAEQAYQB0AGEAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGEAbgB1AHIAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGEAbgB1AHIAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMQBfAF8AMgBfAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAxAF8AXwAyAF8AQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADEAXwBfADIAXwBBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGEAbgB1AHIAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMQBfAF8AMgBfAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBVAG4AaQB0ACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMQBfAF8AMgBfAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADEAXwBfADIAXwBBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4ARgByAG8AbQBNAGEAbgB1AHIAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAxAF8AXwAyAF8AQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAxAF8AXwAyAF8AQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMQBfAF8AMgBfAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwBfAE0AZQB0AGgAbwBkADIAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8ATgAyAE8ARABpAHIAZQBjAHQALgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAzAF8AXwAxAF8ARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBTAG8AaQBsACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAGkAbABfAE4AMgBPAEQAaQByAGUAYwB0AC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMwBfAF8AMQBfAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AUwBvAGkAbABfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBOADIATwBEAGkAcgBlAGMAdAAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADMAXwBfADEAXwBEAGkAcgBlAGMAdABOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFMAbwBpAGwAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8ATgAyAE8ARABpAHIAZQBjAHQALgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAzAF8AXwAxAF8ARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBTAG8AaQBsAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBOADIATwBEAGkAcgBlAGMAdAAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADMAXwBfADEAXwBEAGkAcgBlAGMAdABOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFMAbwBpAGwAXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBOADIATwBEAGkAcgBlAGMAdAAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADMAXwBfADEAXwBEAGkAcgBlAGMAdABOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFMAbwBpAGwAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBOADIATwBEAGkAcgBlAGMAdAAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADMAXwBfADEAXwBEAGkAcgBlAGMAdABOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFMAbwBpAGwAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAGkAbABfAE4AMgBPAEQAaQByAGUAYwB0AC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMwBfAF8AMQBfAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AUwBvAGkAbABfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAGkAbABfAE4AMgBPAEQAaQByAGUAYwB0AC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMwBfAF8AMgBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABlAGQAVABvAFAAYQBzAHQAdQByAGUAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8ATgAyAE8ARABpAHIAZQBjAHQALgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAzAF8AXwAyAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGUAZABUAG8AUABhAHMAdAB1AHIAZQBfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBOADIATwBEAGkAcgBlAGMAdAAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADMAXwBfADIAXwBBAG4AbgB1AGEAbABOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAZQBkAFQAbwBQAGEAcwB0AHUAcgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAGkAbABfAE4AMgBPAEQAaQByAGUAYwB0AC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMwBfAF8AMgBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABlAGQAVABvAFAAYQBzAHQAdQByAGUAXwBVAG4AaQB0ACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAGkAbABfAE4AMgBPAEQAaQByAGUAYwB0AC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8AMwBfAF8AMgBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABlAGQAVABvAFAAYQBzAHQAdQByAGUAXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBOADIATwBEAGkAcgBlAGMAdAAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADMAXwBfADIAXwBBAG4AbgB1AGEAbABOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAZQBkAFQAbwBQAGEAcwB0AHUAcgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8ATgAyAE8ARABpAHIAZQBjAHQALgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAzAF8AXwAyAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGUAZABUAG8AUABhAHMAdAB1AHIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8ATgAyAE8ARABpAHIAZQBjAHQALgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwAzAF8AXwAyAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGUAZABUAG8AUABhAHMAdAB1AHIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAGkAbABfAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANQBfAF8AMQBfAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AUABhAHMAdAB1AHIAZQAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADUAXwBfADEAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFAAYQBzAHQAdQByAGUAXwBUAGkAdABsAGUAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ALgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA1AF8AXwAxAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAGkAbABfAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANQBfAF8AMQBfAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AUABhAHMAdAB1AHIAZQBfAFUAbgBpAHQAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ALgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA1AF8AXwAxAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8AUwBvAHUAcgBjAGUAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ALgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA1AF8AXwAxAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ALgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA1AF8AXwAxAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADUAXwBfADEAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFAAYQBzAHQAdQByAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADUAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0AUABhAHMAdAB1AHIAZQAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADUAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0AUABhAHMAdAB1AHIAZQBfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADUAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0AUABhAHMAdAB1AHIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADUAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0AUABhAHMAdAB1AHIAZQBfAFUAbgBpAHQAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ALgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA1AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAFYAbwBsAGEAdABpAGwAaQBzAGUAZABGAHIAbwBtAFAAYQBzAHQAdQByAGUAXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADUAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0AUABhAHMAdAB1AHIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAGkAbABfAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBWAG8AbABhAHQAaQBsAGkAcwBlAGQARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADUAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAEYAcgBvAG0AUABhAHMAdAB1AHIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAGkAbABfAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADcAXwBfADEAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAGkAbABfAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADcAXwBfADEAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAGkAbABfAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADcAXwBfADEAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAGkAbABfAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADcAXwBfADEAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYALgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA3AF8AXwAxAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAEUAbQBpAHMAcwBpAG8AbgBzAEYAcgBvAG0AUABhAHMAdAB1AHIAZQBfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAGkAbABfAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADcAXwBfADEAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANwBfAF8AMQBfAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBFAG0AaQBzAHMAaQBvAG4AcwBGAHIAbwBtAFAAYQBzAHQAdQByAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAGkAbABfAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADcAXwBfADEAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYARQBtAGkAcwBzAGkAbwBuAHMARgByAG8AbQBQAGEAcwB0AHUAcgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANwBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAbwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANwBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAbwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBUAGkAdABsAGUAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANwBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAbwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANwBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAbwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBVAG4AaQB0ACIALAAiAE0ATQBTAF8ATwB0AGgAZQByAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAGkAbABfAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgAuAFYARQBFAFIARwBfADQAXwA3AF8AMQBfADcAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4ATABvAHMAdABUAG8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAF8AUwBvAHUAcgBjAGUAIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANwBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAbwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAE8AdABoAGUAcgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwBpAGwAXwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYALgBWAEUARQBSAEcAXwA0AF8ANwBfADEAXwA3AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEwAbwBzAHQAVABvAEwAZQBhAGMAaABpAG4AZwBBAG4AZABSAHUAbgBvAGYAZgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIATQBNAFMAXwBPAHQAaABlAHIATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AaQBsAF8ATABlAGEAYwBoAGkAbgBnAEEAbgBkAFIAdQBuAG8AZgBmAC4AVgBFAEUAUgBHAF8ANABfADcAXwAxAF8ANwBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBMAG8AcwB0AFQAbwBMAGUAYQBjAGgAaQBuAGcAQQBuAGQAUgB1AG4AbwBmAGYAXwBBAHIAZwB1AG0AZQBuAHQAcwAiAF0ALAAiAGwAbwBjAGEAbABlACIAOgB7ACIAbABpAHMAdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHIAbwB3AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiADsAIgAsACIAYwBvAGwAdQBtAG4AUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgB0AGgAbwB1AHMAYQBuAGQAcwBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFAAbwBzAGkAdABpAG8AbgBzACIAOgBbADMAXQAsACIAZABlAGMAaQBtAGEAbABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAuACIALAAiAGQAYQB0AGUATwByAGQAZQByACIAOgAiAEQATQBZACIALAAiAGMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbAAiADoAIgAkACIALAAiAGkAcwBDAHUAcgByAGUAbgBjAHkAUwB5AG0AYgBvAGwATABlAGEAZAAiADoAdAByAHUAZQAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAGUAcABCAHkAUwBwAGEAYwBlACIAOgBmAGEAbABzAGUALAAiAHIAbwB3AEwAZQB0AHQAZQByACIAOgAiAFIAIgAsACIAYwBvAGwAdQBtAG4ATABlAHQAdABlAHIAIgA6ACIAQwAiACwAIgByAGMATABlAGYAdABCAHIAYQBjAGsAZQB0ACIAOgAiAFsAIgAsACIAcgBjAFIAaQBnAGgAdABCAHIAYQBjAGsAZQB0ACIAOgAiAF0AIgAsACIAcwB0AGEAdABlAG0AZQBuAHQAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBsAG8AYwBhAGwAZQBOAGEAbQBlACIAOgAiAGUAbgAtAHUAcwAiAH0AfQA=</AFEJSONBlob>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="09eef6d6-daa8-4301-8f9f-b1ec38079286" xsi:nil="true"/>
@@ -30029,7 +30020,24 @@
 </p:properties>
 </file>
 
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{809E3D44-A88D-4EBF-A307-6B8CE77A3361}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -30048,23 +30056,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -30073,4 +30065,12 @@
     <ds:schemaRef ds:uri="7291119c-fce9-4911-96ae-b800be5dccd8"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>